<commit_message>
Şablonlardaki yasal süreler doğrulandı
- TPL-03: KVKK 72 saat (Kurul kararı 2019/10) teyit; 7545 md. 7(1)(b)
  "gecikmeksizin" bildirim, Siber Güvenlik Başkanlığı, md. 16(10) 1–10 M TL
- TPL-06: KVKK md. 9 standart sözleşme 5 iş günü (imza tamamlanmasından),
  Yönetmelik RG 10.07.2024; formda süre kontrol alanı
- TPL-10: EU AI Act takvimi Digital Omnibus (Tüzük (AB) 2026/1744) sonrası:
  Ek III 2 Ara 2027, Ek I 2 Ağu 2028, Art. 50 2 Ağu 2026; yeni yasak satırı
- TPL-13, G-INC-01, G-OVS-01: ilgili [CHECK] işaretleri kaldırıldı
- katalog-onerileri: K-5 (7545), K-6 (EU AI Act)
- Word sürümleri ve inceleme tablosu yeniden üretildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RaFMgY52inRvN44BSaYeeZ
</commit_message>
<xml_diff>
--- a/measurement-tool/output/inceleme-paketi.xlsx
+++ b/measurement-tool/output/inceleme-paketi.xlsx
@@ -748,9 +748,9 @@
       </c>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>KVKK md. 12(5); Kurul kararı 2019/10 (72 saat) [CHECK]
+          <t>KVKK md. 12(5); Kurul kararı 24.01.2019/2019-10 (72 saat)
 GDPR Art. 33
-Law 7545 Siber Güvenlik Kanunu — olay bildirimi [CHECK]
+Law 7545 md. 7(1)(b) (gecikmeksizin bildirim); md. 16(10)
 NIS2 Art. 23
 ISO/IEC 27001:2022 A.5.24–A.5.28
 ISO/IEC 42001 Annex A.8.4 [CHECK]</t>
@@ -1271,7 +1271,7 @@
         <is>
           <t>EU AI Act Art. 14 (high-risk), Art. 26(2)
 GDPR Art. 22
-KVKK md. 11(1)(g) [CHECK]
+KVKK md. 11(1)(g)
 ISO/IEC 42001 Annex A.9 [CHECK sub-control]
 NIST AI RMF GOVERN 3.2</t>
         </is>

</xml_diff>

<commit_message>
Kalan [CHECK] eşlemeleri doğrulandı
- ISO/IEC 42001 Annex A atıfları doğru numaralandırmayla teyit edildi ve
  kontrol adları eklendi (A.7.3, A.10.3, A.4.2, A.8.4, A.9.2); alt kontrol
  belirsizlikleri giderildi (HYG-ING-01 → A.7.2/A.7.6, HYG-ING-04 → A.6.2.4)
- Zayıf atıflar değiştirildi: TRA-ING-01 GDPR Art. 30 → ISO A.6.2.8;
  G-POL-02 AI Act Art. 26(1) ve G-INV-02 ISO A.9.2 kaldırıldı;
  G-RSK-02 NIST MAP 1.5 → MAP 1
- EU AI Act Art. 9, 26(2), 27 kapsamları; DORA Art. 28 / 28(8);
  BDDK Bilgi Sistemleri Yönetmeliği md. 25; KVKK md. 12(2), md. 16;
  SOC 2 CC6.1; TPL-11 GDPR Art. 35(7) asgari içerik
- 02 özeti, şablon README'si, inceleme tablosu ve TPL-11 Word sürümü güncellendi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RaFMgY52inRvN44BSaYeeZ
</commit_message>
<xml_diff>
--- a/measurement-tool/output/inceleme-paketi.xlsx
+++ b/measurement-tool/output/inceleme-paketi.xlsx
@@ -753,7 +753,7 @@
 Law 7545 md. 7(1)(b) (gecikmeksizin bildirim); md. 16(10)
 NIS2 Art. 23
 ISO/IEC 27001:2022 A.5.24–A.5.28
-ISO/IEC 42001 Annex A.8.4 [CHECK]</t>
+ISO/IEC 42001 Annex A.8.4 (communication of incidents)</t>
         </is>
       </c>
       <c r="S2" s="6" t="inlineStr">
@@ -857,9 +857,9 @@
       <c r="R3" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.5.9
-ISO/IEC 42001 Annex A.4 [CHECK sub-control]
+ISO/IEC 42001 Annex A.4.2 (resource documentation)
 NIST AI RMF GOVERN 1.6
-KVKK md. 16 (VERBİS) [CHECK — processing inventory link]
+KVKK md. 16 (VERBİS) ve Veri Sorumluları Sicili Yönetmeliği — kişisel veri işleme envanteri
 GDPR Art. 30</t>
         </is>
       </c>
@@ -965,8 +965,7 @@
       <c r="R4" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.8.15, A.8.16
-KVKK md. 12(1)
-ISO/IEC 42001 Annex A.9.2 [CHECK]</t>
+KVKK md. 12(1)</t>
         </is>
       </c>
       <c r="S4" s="6" t="inlineStr">
@@ -1172,7 +1171,7 @@
       <c r="R6" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 42001 cl. 7.2
-EU AI Act Art. 26(2) [CHECK]
+EU AI Act Art. 26(2) (high-risk deployers)
 ISO/IEC 27001:2022 A.6.3</t>
         </is>
       </c>
@@ -1272,7 +1271,7 @@
           <t>EU AI Act Art. 14 (high-risk), Art. 26(2)
 GDPR Art. 22
 KVKK md. 11(1)(g)
-ISO/IEC 42001 Annex A.9 [CHECK sub-control]
+ISO/IEC 42001 Annex A.9.2 (processes for responsible use)
 NIST AI RMF GOVERN 3.2</t>
         </is>
       </c>
@@ -1485,8 +1484,7 @@
         <is>
           <t>ISO/IEC 27001:2022 A.5.10
 ISO/IEC 42001 Annex A.9.2
-KVKK md. 12(1)
-EU AI Act Art. 26(1) [CHECK — deployer scope]</t>
+KVKK md. 12(1)</t>
         </is>
       </c>
       <c r="S9" s="6" t="inlineStr">
@@ -1696,7 +1694,7 @@
           <t>ISO/IEC 42001 cl. 6.1.2, 8.2
 ISO/IEC 27001:2022 cl. 6.1.2
 NIST AI RMF MAP 1, MANAGE 1
-EU AI Act Art. 9 (high-risk) [CHECK — provider duty]</t>
+EU AI Act Art. 9 (high-risk; provider obligation)</t>
         </is>
       </c>
       <c r="S11" s="6" t="inlineStr">
@@ -1796,7 +1794,7 @@
         <is>
           <t>EU AI Act Art. 6, Annex III
 EU AI Act Art. 50
-NIST AI RMF MAP 1.5 [CHECK]</t>
+NIST AI RMF MAP 1 (context established)</t>
         </is>
       </c>
       <c r="S12" s="6" t="inlineStr">
@@ -1895,9 +1893,9 @@
       <c r="R13" s="6" t="inlineStr">
         <is>
           <t>GDPR Art. 35
-KVKK md. 12(1) [CHECK — no explicit DPIA duty]
+KVKK md. 12(1) (no explicit DPIA duty; risk analysis expected under security measures)
 ISO/IEC 42001 cl. 6.1.4; Annex A.5.2–A.5.4
-EU AI Act Art. 27 (FRIA, where applicable) [CHECK]</t>
+EU AI Act Art. 27 (FRIA: public bodies / public-service providers and Annex III 5(b)-(c) deployers; from 2 Dec 2027)</t>
         </is>
       </c>
       <c r="S13" s="6" t="inlineStr">
@@ -2004,7 +2002,7 @@
 ISO/IEC 27001:2022 A.5.19, A.5.23
 ISO/IEC 42001 Annex A.10.3
 GDPR Art. 28(1), Chapter V
-DORA Art. 28 [CHECK — financial entities]</t>
+DORA Art. 28 (financial entities)</t>
         </is>
       </c>
       <c r="S14" s="6" t="inlineStr">
@@ -2105,8 +2103,8 @@
       <c r="R15" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 9
-DORA Art. 28(8) [CHECK]
-BDDK Bilgi Sistemleri Yönetmeliği — lokalizasyon [CHECK]
+DORA Art. 28(8) (exit strategies)
+BDDK Bankaların Bilgi Sistemleri ve Elektronik Bankacılık Hizmetleri Hakkında Yönetmelik (RG 15.03.2020) md. 25 — birincil ve ikincil sistemler yurt içinde
 ISO/IEC 27001:2022 A.5.23</t>
         </is>
       </c>
@@ -2206,7 +2204,7 @@
       <c r="R16" s="6" t="inlineStr">
         <is>
           <t>GDPR Art. 28(3)
-KVKK md. 9, md. 12(2) [CHECK]
+KVKK md. 9, md. 12(2) (joint responsibility with processor)
 ISO/IEC 27001:2022 A.5.20
 ISO/IEC 42001 Annex A.10.2</t>
         </is>
@@ -2314,7 +2312,7 @@
         <is>
           <t>KVKK md. 9, md. 12(1)
 ISO/IEC 27001:2022 A.8.20, A.8.22
-BDDK Bilgi Sistemleri Yönetmeliği — lokalizasyon [CHECK]</t>
+BDDK Bankaların Bilgi Sistemleri ve Elektronik Bankacılık Hizmetleri Hakkında Yönetmelik (RG 15.03.2020) md. 25 — birincil ve ikincil sistemler yurt içinde</t>
         </is>
       </c>
       <c r="S17" s="6" t="inlineStr">
@@ -2420,7 +2418,7 @@
         <is>
           <t>KVKK md. 9, md. 12(1)
 ISO/IEC 27001:2022 A.5.23, A.8.20
-ISO/IEC 42001 Annex A.10.3 [CHECK]</t>
+ISO/IEC 42001 Annex A.10.3 (suppliers)</t>
         </is>
       </c>
       <c r="S18" s="6" t="inlineStr">
@@ -2525,7 +2523,7 @@
       <c r="R19" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.8.20, A.5.14
-ISO/IEC 42001 Annex A.7.3 [CHECK]
+ISO/IEC 42001 Annex A.7.3 (acquisition of data)
 KVKK md. 12(1)
 NIS2 Art. 21(2)</t>
         </is>
@@ -2946,7 +2944,7 @@
 KVKK md. 6
 GDPR Art. 5(1)(c)
 GDPR Art. 25(1)
-ISO/IEC 42001 Annex A.7 [CHECK sub-control]</t>
+ISO/IEC 42001 Annex A.7.2, A.7.6 (data for development; data preparation)</t>
         </is>
       </c>
       <c r="S23" s="6" t="inlineStr">
@@ -3256,8 +3254,8 @@
       <c r="R26" s="6" t="inlineStr">
         <is>
           <t>GDPR Art. 32(1)(d)
-NIST AI RMF MEASURE 2.10 [CHECK]
-ISO/IEC 42001 Annex A.7 [CHECK sub-control]</t>
+NIST AI RMF MEASURE 2.10 (privacy risk examined and documented)
+ISO/IEC 42001 Annex A.6.2.4 (verification and validation)</t>
         </is>
       </c>
       <c r="S26" s="6" t="inlineStr">
@@ -3465,7 +3463,7 @@
         <is>
           <t>ISO/IEC 27001:2022 A.5.16, A.5.17, A.8.5
 KVKK md. 12(1)
-SOC 2 CC6.1 [CHECK]</t>
+SOC 2 CC6.1</t>
         </is>
       </c>
       <c r="S28" s="6" t="inlineStr">
@@ -3677,7 +3675,7 @@
         <is>
           <t>ISO/IEC 27001:2022 A.8.15
 ISO/IEC 42001 Annex A.7.5
-GDPR Art. 30 [CHECK — records link]
+ISO/IEC 42001 Annex A.6.2.8 (recording of event logs)
 KVKK md. 12(1)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
A2 pilot: kontrol listesi + sabit puanlama kuralı (G-POL-02, HYG-ING-02)
- schema.md 5.5: checks alanı, kontrol türleri, ölçüm tipleri, sabit kural, örneklem
- source/terms.yaml: 7 terim tanımı
- tools/kontrol.py: puan hesabı ve rubric metni üretimi (tek yer)
- qs.py: rehberde kontrol tablosu + terimler; CSV'de kontrol başına satır; seviye puanı kontrollerden hesaplar
- inceleme.py: rubric üretilmiş metinden, yeni Kontroller sütunu
- G-POL-02, HYG-ING-02 çevrildi; çıktılar yeniden üretildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RaFMgY52inRvN44BSaYeeZ
</commit_message>
<xml_diff>
--- a/measurement-tool/output/inceleme-paketi.xlsx
+++ b/measurement-tool/output/inceleme-paketi.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maddeler" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Maddeler'!$A$1:$V$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Maddeler'!$A$1:$W$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -508,7 +508,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5. EN metinler U–V sütunlarında gizli (grup "+" ile açılır). TR ile anlam farkı görürsen yorumda belirt.</t>
+          <t>5. EN metinler V–W sütunlarında gizli (grup "+" ile açılır). TR ile anlam farkı görürsen yorumda belirt.</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V30"/>
+  <dimension ref="A1:W30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -548,12 +548,13 @@
     <col width="45" customWidth="1" min="13" max="13"/>
     <col width="45" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="45" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
-    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="21" max="22"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="40" customWidth="1" min="21" max="21"/>
+    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="22" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -634,35 +635,40 @@
       </c>
       <c r="P1" s="3" t="inlineStr">
         <is>
+          <t>Kontroller</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
           <t>Gözden geçirme (ay)</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Kanıt</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Eşleme</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Servisler</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Not (iç)</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Title (EN)</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>Rubric 2 (EN)</t>
         </is>
@@ -736,17 +742,18 @@
           <t>2'yi karşılıyor; her tatbikat ya da olaydan çıkan dersler kayıtlı, aksiyonlar kapanışa kadar izleniyor ve prosedür 12 ay içinde gözden geçirilmiş.</t>
         </is>
       </c>
-      <c r="P2" s="6" t="n">
+      <c r="P2" s="6" t="inlineStr"/>
+      <c r="Q2" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q2" s="6" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
         <is>
           <t>[DOC] En az şu AI olay türlerini adlandıran prosedür — prompt ya da çıktı yoluyla veri sızıntısı, etkisi olan zararlı ya da yanlış çıktı, model üzerinden yetkisiz erişim, sağlayıcı tarafı olay
 [DOC] Bildirim süreleri tablosu (ör. KVKK ihlal bildirimi, sektör ve siber güvenlik yükümlülükleri)
 [TST] Bir tatbikatın ya da ele alınmış bir AI olayının kaydı</t>
         </is>
       </c>
-      <c r="R2" s="6" t="inlineStr">
+      <c r="S2" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 12(5); Kurul kararı 24.01.2019/2019-10 (72 saat)
 GDPR Art. 33
@@ -756,22 +763,22 @@
 ISO/IEC 42001 Annex A.8.4 (communication of incidents)</t>
         </is>
       </c>
-      <c r="S2" s="6" t="inlineStr">
+      <c r="T2" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, SU-05</t>
         </is>
       </c>
-      <c r="T2" s="6" t="inlineStr">
+      <c r="U2" s="6" t="inlineStr">
         <is>
           <t>SU-05 bu maddeyi kapatan hizmet.</t>
         </is>
       </c>
-      <c r="U2" s="6" t="inlineStr">
+      <c r="V2" s="6" t="inlineStr">
         <is>
           <t>AI incident procedure</t>
         </is>
       </c>
-      <c r="V2" s="6" t="inlineStr">
+      <c r="W2" s="6" t="inlineStr">
         <is>
           <t>The procedure names the four incident types, the reporting chain with named roles and the applicable deadlines, is linked to the general process, and an exercise or a handled AI incident is recorded in the last 12 months.</t>
         </is>
@@ -845,16 +852,17 @@
           <t>2'yi karşılıyor ve envanter 6 ay içinde G-INV-02 trafik verileriyle karşılaştırılmış; eklenen ve çıkarılan kayıtların tarihli kaydı var.</t>
         </is>
       </c>
-      <c r="P3" s="6" t="n">
+      <c r="P3" s="6" t="inlineStr"/>
+      <c r="Q3" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
         <is>
           <t>[DOC] Amaç, sahip, kullanıcılar, veri kategorileri, sağlayıcı, profil ve durum alanlarını içeren envanter
 [DOC] Karşılaştırma için onaylı araç listesi (G-POL-02) ve satın alma ya da proje kayıtları</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
+      <c r="S3" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.5.9
 ISO/IEC 42001 Annex A.4.2 (resource documentation)
@@ -863,22 +871,22 @@
 GDPR Art. 30</t>
         </is>
       </c>
-      <c r="S3" s="6" t="inlineStr">
+      <c r="T3" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-04, SU-01</t>
         </is>
       </c>
-      <c r="T3" s="6" t="inlineStr">
+      <c r="U3" s="6" t="inlineStr">
         <is>
           <t>Envanter, AS-02 kapsamının (hangi sistemler matrisle ölçülecek) girdisi. Profil alanı CE/SOV/hibrit: hibrit sistemde iki profil de ayrı ölçülür.</t>
         </is>
       </c>
-      <c r="U3" s="6" t="inlineStr">
+      <c r="V3" s="6" t="inlineStr">
         <is>
           <t>AI system inventory</t>
         </is>
       </c>
-      <c r="V3" s="6" t="inlineStr">
+      <c r="W3" s="6" t="inlineStr">
         <is>
           <t>Every entry has all required fields, no system found in procurement records, the sanctioned tool list or interviews is missing, and the inventory was updated in the last 6 months.</t>
         </is>
@@ -952,38 +960,39 @@
           <t>2'yi karşılıyor; raporlar 3 ay içinde gözden geçiriliyor ve onaylı listede (G-POL-02) olmayan servislere giden trafik kayıtlı bir takip başlatıyor.</t>
         </is>
       </c>
-      <c r="P4" s="6" t="n">
+      <c r="P4" s="6" t="inlineStr"/>
+      <c r="Q4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Q4" s="6" t="inlineStr">
+      <c r="R4" s="6" t="inlineStr">
         <is>
           <t>[CFG] DNS, proxy ya da firewall kayıt yapılandırması ve saklama süresi
 [DOC] Tanımlama için kullanılan, güncelleme tarihli AI servis alan adı/uç nokta listesi
 [LOG] En az 30 günlük dönem için birim bazında AI servis trafiği raporu ya da sorgu sonucu</t>
         </is>
       </c>
-      <c r="R4" s="6" t="inlineStr">
+      <c r="S4" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.8.15, A.8.16
 KVKK md. 12(1)</t>
         </is>
       </c>
-      <c r="S4" s="6" t="inlineStr">
+      <c r="T4" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-04, SU-01</t>
         </is>
       </c>
-      <c r="T4" s="6" t="inlineStr">
+      <c r="U4" s="6" t="inlineStr">
         <is>
           <t>AS-04'ün ölçüm aracındaki karşılığı. Yalnız üst veri; içerik incelemesi bu madde kapsamında değil. CE'de L1 çünkü veri dışarıya bu kanaldan çıkıyor; SOV'da L2. 90 gün eşiği mevzuat şartı değil, operasyonel tercih — pilotta kalibre edilecek.</t>
         </is>
       </c>
-      <c r="U4" s="6" t="inlineStr">
+      <c r="V4" s="6" t="inlineStr">
         <is>
           <t>Visibility of AI service use</t>
         </is>
       </c>
-      <c r="V4" s="6" t="inlineStr">
+      <c r="W4" s="6" t="inlineStr">
         <is>
           <t>Logs are retained for at least 90 days, traffic is attributable to a unit or user group, the AI service domain list was updated in the last 6 months, and a report covering at least 30 days can be produced on request.</t>
         </is>
@@ -1057,16 +1066,17 @@
           <t>2'yi karşılıyor; içerik 12 ay içinde güncellenmiş ve anlama ölçülüyor (sınav ya da uygulama), sonuçlar kayıtlı.</t>
         </is>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="P5" s="6" t="inlineStr"/>
+      <c r="Q5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q5" s="6" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr">
         <is>
           <t>[DOC] Üç konuyu kapsayan program içeriği
 [LOG] Kişi başına tarihli tamamlama kayıtları; payda için G-INV-01'den AI kullanıcı sayısı</t>
         </is>
       </c>
-      <c r="R5" s="6" t="inlineStr">
+      <c r="S5" s="6" t="inlineStr">
         <is>
           <t>EU AI Act Art. 4
 ISO/IEC 42001 cl. 7.3
@@ -1074,22 +1084,22 @@
 NIST AI RMF GOVERN 2.2</t>
         </is>
       </c>
-      <c r="S5" s="6" t="inlineStr">
+      <c r="T5" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, EN-02</t>
         </is>
       </c>
-      <c r="T5" s="6" t="inlineStr">
+      <c r="U5" s="6" t="inlineStr">
         <is>
           <t>%80 ve 60 gün eşikleri ölçütü sayılabilir kılmak için konuldu; pilotta kalibre edilecek. EN-02 bu maddeyi kapatan hizmet.</t>
         </is>
       </c>
-      <c r="U5" s="6" t="inlineStr">
+      <c r="V5" s="6" t="inlineStr">
         <is>
           <t>AI literacy for all users</t>
         </is>
       </c>
-      <c r="V5" s="6" t="inlineStr">
+      <c r="W5" s="6" t="inlineStr">
         <is>
           <t>The programme covers the three topics and at least 80% of AI users have a recorded completion; new users complete it within 60 days of access.</t>
         </is>
@@ -1159,34 +1169,35 @@
           <t>2'yi karşılıyor ve rol sahipleri 12 ay içinde tazeleme eğitimini tamamlamış.</t>
         </is>
       </c>
-      <c r="P6" s="6" t="n">
+      <c r="P6" s="6" t="inlineStr"/>
+      <c r="Q6" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q6" s="6" t="inlineStr">
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>[DOC] Eğitim modülleriyle eşlenmiş AI rolleri listesi (G-ROL-01 ve G-OVS-01'den)
 [LOG] Rol sahibi başına tamamlama kayıtları</t>
         </is>
       </c>
-      <c r="R6" s="6" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 42001 cl. 7.2
 EU AI Act Art. 26(2) (high-risk deployers)
 ISO/IEC 27001:2022 A.6.3</t>
         </is>
       </c>
-      <c r="S6" s="6" t="inlineStr">
+      <c r="T6" s="6" t="inlineStr">
         <is>
           <t>AS-02, EN-03</t>
         </is>
       </c>
-      <c r="T6" s="6" t="inlineStr"/>
-      <c r="U6" s="6" t="inlineStr">
+      <c r="U6" s="6" t="inlineStr"/>
+      <c r="V6" s="6" t="inlineStr">
         <is>
           <t>Role-based training</t>
         </is>
       </c>
-      <c r="V6" s="6" t="inlineStr">
+      <c r="W6" s="6" t="inlineStr">
         <is>
           <t>Every AI role is mapped to a module and every current role holder has a recorded completion.</t>
         </is>
@@ -1256,17 +1267,18 @@
           <t>2'yi karşılıyor ve 6 ay içinde süre sınırında tamamlanan incelemelerin oranı sistem başına ölçülmüş ve kaydedilmiş.</t>
         </is>
       </c>
-      <c r="P7" s="6" t="n">
+      <c r="P7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q7" s="6" t="inlineStr">
+      <c r="R7" s="6" t="inlineStr">
         <is>
           <t>[DOC] Sistem başına dört unsuru (çıktı sınıfları, inceleyen rol, süre sınırı, bekleme durumu) içeren gözetim prosedürü
 [TST] Sistem başına en az bir uçtan uca işletim kaydı (gerçek vaka ya da test)
 [LOG] Kararları ve süreleri gösteren inceleme kuyruğu kayıtları</t>
         </is>
       </c>
-      <c r="R7" s="6" t="inlineStr">
+      <c r="S7" s="6" t="inlineStr">
         <is>
           <t>EU AI Act Art. 14 (high-risk), Art. 26(2)
 GDPR Art. 22
@@ -1275,22 +1287,22 @@
 NIST AI RMF GOVERN 3.2</t>
         </is>
       </c>
-      <c r="S7" s="6" t="inlineStr">
+      <c r="T7" s="6" t="inlineStr">
         <is>
           <t>AS-02, DS-03, AU-03</t>
         </is>
       </c>
-      <c r="T7" s="6" t="inlineStr">
+      <c r="U7" s="6" t="inlineStr">
         <is>
           <t>v0'da L3 "process gap" notu + L5 artefaktıydı. Uçtan uca işletim şartı 2'ye kondu: kâğıt üzerindeki prosedür L3 kapısını açmaz. BEH-RES escalation bu maddeye bağlanır.</t>
         </is>
       </c>
-      <c r="U7" s="6" t="inlineStr">
+      <c r="V7" s="6" t="inlineStr">
         <is>
           <t>Human oversight</t>
         </is>
       </c>
-      <c r="V7" s="6" t="inlineStr">
+      <c r="W7" s="6" t="inlineStr">
         <is>
           <t>Every system has the four elements defined (or a signed no-review decision), and each system with defined review classes has at least one recorded end-to-end run.</t>
         </is>
@@ -1364,16 +1376,17 @@
           <t>2'yi karşılıyor ve politika 12 ay içinde gözden geçirilmiş; değişiklikleri ya da değişiklik olmadığını belirten tarihli kayıt var.</t>
         </is>
       </c>
-      <c r="P8" s="6" t="n">
+      <c r="P8" s="6" t="inlineStr"/>
+      <c r="Q8" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q8" s="6" t="inlineStr">
+      <c r="R8" s="6" t="inlineStr">
         <is>
           <t>[DOC] Onay kaydıyla (onaylayan, tarih, sürüm) yapay zekâ politikası
 [DOC] Duyuru kaydı (intranet yayını, e-posta, okundu listesi)</t>
         </is>
       </c>
-      <c r="R8" s="6" t="inlineStr">
+      <c r="S8" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 42001 cl. 5.2
 ISO/IEC 42001 Annex A.2.2, A.2.4
@@ -1381,22 +1394,22 @@
 NIST AI RMF GOVERN 1.2</t>
         </is>
       </c>
-      <c r="S8" s="6" t="inlineStr">
+      <c r="T8" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, DS-03, SU-01</t>
         </is>
       </c>
-      <c r="T8" s="6" t="inlineStr">
+      <c r="U8" s="6" t="inlineStr">
         <is>
           <t>AI'nin bilgi güvenliği politikası içinde ayrı bir bölüm olarak ele alınması da kabul edilir; ölçüt içerik, belge adı değil. DS-03 bu maddeyi kapatan hizmet.</t>
         </is>
       </c>
-      <c r="U8" s="6" t="inlineStr">
+      <c r="V8" s="6" t="inlineStr">
         <is>
           <t>AI policy</t>
         </is>
       </c>
-      <c r="V8" s="6" t="inlineStr">
+      <c r="W8" s="6" t="inlineStr">
         <is>
           <t>The policy is approved by top management or a delegated body, names the accountable role, defines the approval route for new AI systems, references G-POL-02, and a record shows it was communicated to all staff in scope.</t>
         </is>
@@ -1452,59 +1465,69 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>Çalışanların AI araçlarını kullanımına dair yazılı kural yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>Kurallar var ama şunlardan en az biri geçerli: kurumun veri sınıflandırmasına atıf yapmıyor; onaylı araç listesi yok; liste son 12 ayda güncellenmemiş; görüşülen çalışanlar kuralları bilmiyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>Kurallar veri sınıflandırmasına atıf yapıyor; onaylı araç listesi araç başına izin verilen veri sınıflarını belirtiyor ve son 12 ayda güncellenmiş; farklı birimlerden görüşülen en az iki çalışan kuralları tutarlı anlatıyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve kurallara uyum 6 ay içinde G-INV-02 verileriyle karşılaştırılarak kontrol edilmiş; bulgu ve aksiyonların tarihli kaydı var.</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="n">
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Çalışanların yapay zekâ araçlarını kullanımına dair yazılı kural var (ayrı belge ya da bir politikanın içinde).
+c2 [temel] Kurallar kurumun veri sınıflarına atıf yapıyor.
+c3 [temel] Onaylı araç listesi var ve listedeki her araç için izin verilen veri sınıfları yazılı.
+c4 [temel] Onaylı araç listesinin son güncelleme tarihi son 12 ay içinde. [≤ 12 ay]
+c5 [temel, QS dışı] Farklı birimlerden iki çalışana "hangi yapay zekâ aracını kullanabilirsin, ona &lt;bir veri sınıfı&gt; girebilir misin?" diye sorulduğunda cevapları listeyle uyuşuyor. [2/2]
+s1 [sürdürme] Kurallara uyum G-INV-02 kullanım verisiyle karşılaştırılmış ve bu karşılaştırmanın tarihli kaydı 6 ay içinde. [≤ 6 ay]</t>
+        </is>
+      </c>
+      <c r="Q9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q9" s="6" t="inlineStr">
+      <c r="R9" s="6" t="inlineStr">
         <is>
           <t>[DOC] Kabul edilebilir kullanım kuralları (ayrı belge ya da AI/kabul edilebilir kullanım politikası içinde)
 [DOC] Araç başına izin verilen veri sınıflarını ve son güncelleme tarihini gösteren onaylı AI araç listesi
-[INT] Farklı birimlerden en az iki çalışan kuralları tutarlı biçimde anlatıyor</t>
-        </is>
-      </c>
-      <c r="R9" s="6" t="inlineStr">
+[INT] Farklı birimlerden iki çalışanın hangi aracı kullanabileceği ve hangi veri sınıfını girebileceğine dair cevapları (kontrol c5)</t>
+        </is>
+      </c>
+      <c r="S9" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.5.10
 ISO/IEC 42001 Annex A.9.2
 KVKK md. 12(1)</t>
         </is>
       </c>
-      <c r="S9" s="6" t="inlineStr">
+      <c r="T9" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-04, DS-03, EN-02</t>
         </is>
       </c>
-      <c r="T9" s="6" t="inlineStr">
+      <c r="U9" s="6" t="inlineStr">
         <is>
           <t>L0: dış araçlara veri girişi teknik kontrol kurulmadan da başlar; kuralın olmaması kurumun her profilde ilk açığı. Kurumun veri sınıflandırması yoksa 1'in üstüne çıkmaz.</t>
         </is>
       </c>
-      <c r="U9" s="6" t="inlineStr">
+      <c r="V9" s="6" t="inlineStr">
         <is>
           <t>Acceptable use of AI tools</t>
         </is>
       </c>
-      <c r="V9" s="6" t="inlineStr">
-        <is>
-          <t>Rules refer to the data classification, a sanctioned tool list states the allowed data classes per tool and was updated in the last 12 months, and at least two interviewed staff from different units describe the rules consistently.</t>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -1576,17 +1599,18 @@
           <t>2'yi karşılıyor ve sahipler ile rol atamaları 12 ay içinde teyit edilmiş; personel değişikliği sonrası güncellemeleri de içeren tarihli kayıt var.</t>
         </is>
       </c>
-      <c r="P10" s="6" t="n">
+      <c r="P10" s="6" t="inlineStr"/>
+      <c r="Q10" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q10" s="6" t="inlineStr">
+      <c r="R10" s="6" t="inlineStr">
         <is>
           <t>[DOC] G-INV-01'de kişi ya da rol adıyla doldurulmuş sahip alanı
 [DOC] AI yönetişim rolü için atama yazısı ya da görev tanımı
 [DOC] DPO ve güvenlik için tanımlı danışma noktaları (ör. yeni sistem, yeni veri kategorisi, yeni sağlayıcı)</t>
         </is>
       </c>
-      <c r="R10" s="6" t="inlineStr">
+      <c r="S10" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 42001 cl. 5.3
 ISO/IEC 42001 Annex A.3.2
@@ -1594,18 +1618,18 @@
 NIST AI RMF GOVERN 2.1</t>
         </is>
       </c>
-      <c r="S10" s="6" t="inlineStr">
+      <c r="T10" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, DS-03</t>
         </is>
       </c>
-      <c r="T10" s="6" t="inlineStr"/>
-      <c r="U10" s="6" t="inlineStr">
+      <c r="U10" s="6" t="inlineStr"/>
+      <c r="V10" s="6" t="inlineStr">
         <is>
           <t>Roles and accountability</t>
         </is>
       </c>
-      <c r="V10" s="6" t="inlineStr">
+      <c r="W10" s="6" t="inlineStr">
         <is>
           <t>Every inventoried system has a named owner, the governance role is formally assigned, consultation points are defined, and at least one record shows a consultation took place (or none was triggered in the last 12 months, stated).</t>
         </is>
@@ -1679,17 +1703,18 @@
           <t>2'yi karşılıyor ve her değerlendirme 12 ay içinde ya da her tetikleyici olaydan sonra (hangisi önce gelirse) tekrarlanmış, kayıtları var.</t>
         </is>
       </c>
-      <c r="P11" s="6" t="n">
+      <c r="P11" s="6" t="inlineStr"/>
+      <c r="Q11" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q11" s="6" t="inlineStr">
+      <c r="R11" s="6" t="inlineStr">
         <is>
           <t>[DOC] AI'ye özgü riskleri kapsayan risk değerlendirme yöntemi (kriterler, ölçekler, kabul)
 [DOC] Envanterdeki her sistem için tarihli, muamele kararlarını ve sahip onayını içeren risk değerlendirmesi
 [DOC] Tanımlı yeniden değerlendirme tetikleyicileri (yeni model ya da sağlayıcı, yeni veri kategorisi, yeni kullanıcı grubu, olay)</t>
         </is>
       </c>
-      <c r="R11" s="6" t="inlineStr">
+      <c r="S11" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 42001 cl. 6.1.2, 8.2
 ISO/IEC 27001:2022 cl. 6.1.2
@@ -1697,22 +1722,22 @@
 EU AI Act Art. 9 (high-risk; provider obligation)</t>
         </is>
       </c>
-      <c r="S11" s="6" t="inlineStr">
+      <c r="T11" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-07, SU-01</t>
         </is>
       </c>
-      <c r="T11" s="6" t="inlineStr">
+      <c r="U11" s="6" t="inlineStr">
         <is>
           <t>Dört AI risk grubu sabit liste olarak verildi ki "AI'ye özgü" ölçütü yoruma kalmasın. Kurum ISO 27001 risk yöntemini kullanıyorsa ve dört grup içindeyse kabul edilir.</t>
         </is>
       </c>
-      <c r="U11" s="6" t="inlineStr">
+      <c r="V11" s="6" t="inlineStr">
         <is>
           <t>AI risk assessment</t>
         </is>
       </c>
-      <c r="V11" s="6" t="inlineStr">
+      <c r="W11" s="6" t="inlineStr">
         <is>
           <t>Every production system has a dated assessment made with the written method that addresses the four AI-specific risk groups, with treatment decisions signed off by the owner, and re-assessment triggers are defined.</t>
         </is>
@@ -1782,37 +1807,38 @@
           <t>2'yi karşılıyor ve sınıflandırmalar 12 ay içinde ve her amaç ya da kullanıcı grubu değişikliğinden sonra yeniden teyit edilmiş, kayıtları var.</t>
         </is>
       </c>
-      <c r="P12" s="6" t="n">
+      <c r="P12" s="6" t="inlineStr"/>
+      <c r="Q12" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q12" s="6" t="inlineStr">
+      <c r="R12" s="6" t="inlineStr">
         <is>
           <t>[DOC] Sistem başına kategori, ölçütlere atıf yapan gerekçe, imzalayan ve tarih içeren sınıflandırma kaydı</t>
         </is>
       </c>
-      <c r="R12" s="6" t="inlineStr">
+      <c r="S12" s="6" t="inlineStr">
         <is>
           <t>EU AI Act Art. 6, Annex III
 EU AI Act Art. 50
 NIST AI RMF MAP 1 (context established)</t>
         </is>
       </c>
-      <c r="S12" s="6" t="inlineStr">
+      <c r="T12" s="6" t="inlineStr">
         <is>
           <t>AS-02, AU-03</t>
         </is>
       </c>
-      <c r="T12" s="6" t="inlineStr">
+      <c r="U12" s="6" t="inlineStr">
         <is>
           <t>v0'da L5 artefaktıydı. L3'e çekildi: hangi yükümlülüklerin uygulanacağını bu karar belirliyor, L5'i beklemek geç. Hukuki yorum gerekirse hukuk ortağı; Lecta kararı vermez, kayıt ve gerekçenin varlığını ölçer.</t>
         </is>
       </c>
-      <c r="U12" s="6" t="inlineStr">
+      <c r="V12" s="6" t="inlineStr">
         <is>
           <t>AI risk classification</t>
         </is>
       </c>
-      <c r="V12" s="6" t="inlineStr">
+      <c r="W12" s="6" t="inlineStr">
         <is>
           <t>Every inventoried system has a classification with rationale referencing the criteria, applicable sector rules are considered, and a named person signed it.</t>
         </is>
@@ -1882,15 +1908,16 @@
           <t>2'yi karşılıyor; önlemler kapanışa kadar izleniyor ve her değerlendirme 12 ay içinde ya da veri kategorisi veya sağlayıcı değişikliğinden sonra güncellenmiş.</t>
         </is>
       </c>
-      <c r="P13" s="6" t="n">
+      <c r="P13" s="6" t="inlineStr"/>
+      <c r="Q13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q13" s="6" t="inlineStr">
+      <c r="R13" s="6" t="inlineStr">
         <is>
           <t>[DOC] Sistem başına, pipeline aşamalarında veri haritası, risk listesi, önlemler ve DPO görüşünü içeren etki değerlendirmesi</t>
         </is>
       </c>
-      <c r="R13" s="6" t="inlineStr">
+      <c r="S13" s="6" t="inlineStr">
         <is>
           <t>GDPR Art. 35
 KVKK md. 12(1) (no explicit DPIA duty; risk analysis expected under security measures)
@@ -1898,22 +1925,22 @@
 EU AI Act Art. 27 (FRIA: public bodies / public-service providers and Annex III 5(b)-(c) deployers; from 2 Dec 2027)</t>
         </is>
       </c>
-      <c r="S13" s="6" t="inlineStr">
+      <c r="T13" s="6" t="inlineStr">
         <is>
           <t>AS-02, AS-07</t>
         </is>
       </c>
-      <c r="T13" s="6" t="inlineStr">
+      <c r="U13" s="6" t="inlineStr">
         <is>
           <t>AS-07 çekirdek çıktısı bu maddeyi 2'ye taşır. Hukuki sonuç (hukuka uygunluk sebebi, aktarım mekanizması) bu maddenin ölçütü değil; o kısım hukuk ortağında.</t>
         </is>
       </c>
-      <c r="U13" s="6" t="inlineStr">
+      <c r="V13" s="6" t="inlineStr">
         <is>
           <t>Impact assessment for personal data</t>
         </is>
       </c>
-      <c r="V13" s="6" t="inlineStr">
+      <c r="W13" s="6" t="inlineStr">
         <is>
           <t>Every AI system processing personal data has an assessment with a data map across all pipeline stages, identified cross-border points, mitigations with owners, and a recorded DPO opinion.</t>
         </is>
@@ -1987,16 +2014,17 @@
           <t>2'yi karşılıyor ve her değerlendirme 12 ay içinde ve sağlayıcı koşullarında ya da alt işleyenlerde bildirilen her değişiklikten sonra tekrarlanmış, kayıtları var.</t>
         </is>
       </c>
-      <c r="P14" s="6" t="n">
+      <c r="P14" s="6" t="inlineStr"/>
+      <c r="Q14" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q14" s="6" t="inlineStr">
+      <c r="R14" s="6" t="inlineStr">
         <is>
           <t>[DOC] Sağlayıcı başına beş konuyu kapsayan, ilk kullanımdan önce tarihli değerlendirme kaydı
 [DOC] Dayanılan sağlayıcı belgeleri (koşullar, veri işleme eki, alt işleyen listesi, veri yerleşimi beyanı)</t>
         </is>
       </c>
-      <c r="R14" s="6" t="inlineStr">
+      <c r="S14" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 9 (Law 7499 amendment)
 ISO/IEC 27001:2022 A.5.19, A.5.23
@@ -2005,22 +2033,22 @@
 DORA Art. 28 (financial entities)</t>
         </is>
       </c>
-      <c r="S14" s="6" t="inlineStr">
+      <c r="T14" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-07, DS-04</t>
         </is>
       </c>
-      <c r="T14" s="6" t="inlineStr">
+      <c r="U14" s="6" t="inlineStr">
         <is>
           <t>CE profilinin çekirdek maddesi, bu yüzden CE'de L1. v0'da ATT-ING (L4) içindeydi. Hukuki yeterlilik (aktarım mekanizmasının geçerliliği) hukuk ortağında; bu madde değerlendirmenin yapılıp yapılmadığını ve kapsamını ölçer.</t>
         </is>
       </c>
-      <c r="U14" s="6" t="inlineStr">
+      <c r="V14" s="6" t="inlineStr">
         <is>
           <t>AI provider assessment before use</t>
         </is>
       </c>
-      <c r="V14" s="6" t="inlineStr">
+      <c r="W14" s="6" t="inlineStr">
         <is>
           <t>Every provider used with organisational data has an assessment covering all five topics, dated before first use, with the provider documents relied on retained.</t>
         </is>
@@ -2090,17 +2118,18 @@
           <t>2'yi karşılıyor ve en az bir kritik sağlayıcının çıkış planı 12 ay içinde işletilmiş (masa başı ya da teknik test), kaydı var.</t>
         </is>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="P15" s="6" t="inlineStr"/>
+      <c r="Q15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q15" s="6" t="inlineStr">
+      <c r="R15" s="6" t="inlineStr">
         <is>
           <t>[DOC] Sağlayıcı başına üç soruyu kaynaklarıyla (şirket sicili, sözleşmeler, mimari belgeler) cevaplayan kayıt
 [DOC] Kritik olarak nitelenen her sağlayıcı için çıkış planı ya da alternatif sağlayıcı değerlendirmesi
 [LOG] Sınır sorusu için çıkış trafiği ya da veri yerleşimi kanıtı (yalnız sağlayıcı beyanı değil)</t>
         </is>
       </c>
-      <c r="R15" s="6" t="inlineStr">
+      <c r="S15" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 9
 DORA Art. 28(8) (exit strategies)
@@ -2108,22 +2137,22 @@
 ISO/IEC 27001:2022 A.5.23</t>
         </is>
       </c>
-      <c r="S15" s="6" t="inlineStr">
+      <c r="T15" s="6" t="inlineStr">
         <is>
           <t>AS-02, DS-04</t>
         </is>
       </c>
-      <c r="T15" s="6" t="inlineStr">
+      <c r="U15" s="6" t="inlineStr">
         <is>
           <t>AS-05'ten gelen egemenlik testi (S-11). SOV'da L1: egemenlik iddiasının kendisi bu üç soruya dayanıyor. "Kritik sağlayıcı" tanımı değerlendirme kaydında kurum tarafından yapılır; tanım yoksa 2 verilmez.</t>
         </is>
       </c>
-      <c r="U15" s="6" t="inlineStr">
+      <c r="V15" s="6" t="inlineStr">
         <is>
           <t>Sovereignty test</t>
         </is>
       </c>
-      <c r="V15" s="6" t="inlineStr">
+      <c r="W15" s="6" t="inlineStr">
         <is>
           <t>All three questions are answered with sources for every provider in scope, the boundary answer is supported by egress or residency evidence, and every critical provider has an exit plan or an alternative-provider assessment.</t>
         </is>
@@ -2193,15 +2222,16 @@
           <t>2'yi karşılıyor ve sağlayıcı koşul değişiklikleri izleniyor: her sağlayıcı için koşulların 12 ay içinde yeniden kontrol edildiğini gösteren kayıt var.</t>
         </is>
       </c>
-      <c r="P16" s="6" t="n">
+      <c r="P16" s="6" t="inlineStr"/>
+      <c r="Q16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q16" s="6" t="inlineStr">
+      <c r="R16" s="6" t="inlineStr">
         <is>
           <t>[DOC] Sağlayıcı başına, beş madde işaretlenmiş sözleşme ya da kabul edilmiş koşullar</t>
         </is>
       </c>
-      <c r="R16" s="6" t="inlineStr">
+      <c r="S16" s="6" t="inlineStr">
         <is>
           <t>GDPR Art. 28(3)
 KVKK md. 9, md. 12(2) (joint responsibility with processor)
@@ -2209,22 +2239,22 @@
 ISO/IEC 42001 Annex A.10.2</t>
         </is>
       </c>
-      <c r="S16" s="6" t="inlineStr">
+      <c r="T16" s="6" t="inlineStr">
         <is>
           <t>AS-02, DS-04</t>
         </is>
       </c>
-      <c r="T16" s="6" t="inlineStr">
+      <c r="U16" s="6" t="inlineStr">
         <is>
           <t>Hukuki yeterlilik değil maddelerin varlığı ölçülür. Tıkla-kabul SaaS koşulları da "sözleşme" sayılır; kurum pazarlık edemiyorsa risk kabulü yolu açık.</t>
         </is>
       </c>
-      <c r="U16" s="6" t="inlineStr">
+      <c r="V16" s="6" t="inlineStr">
         <is>
           <t>Contractual safeguards with AI providers</t>
         </is>
       </c>
-      <c r="V16" s="6" t="inlineStr">
+      <c r="W16" s="6" t="inlineStr">
         <is>
           <t>Every provider used with organisational data has all five clauses, or each missing clause has a risk acceptance signed by the system owner and referenced in G-RSK-01.</t>
         </is>
@@ -2298,39 +2328,40 @@
           <t>2'yi karşılıyor; çıkarım ortamından dışarıya bağlantı denemeleri alarm üretiyor ve ele alınıyor; çıkış testi 6 ay içinde tekrarlanıyor.</t>
         </is>
       </c>
-      <c r="P17" s="6" t="n">
+      <c r="P17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q17" s="6" t="inlineStr">
+      <c r="R17" s="6" t="inlineStr">
         <is>
           <t>[DOC] Her modelin nerede çalıştığını ve sınırı gösteren mimari
 [CFG] Çıkarım ortamı için çıkış politikası (varsayılan red, listelenmiş iç hedefler)
 [LOG] Çıkarım ortamından en az 7 günlük çalışmaya ait çıkış/düşürme kayıtları ya da tarihli çıkış testi</t>
         </is>
       </c>
-      <c r="R17" s="6" t="inlineStr">
+      <c r="S17" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 9, md. 12(1)
 ISO/IEC 27001:2022 A.8.20, A.8.22
 BDDK Bankaların Bilgi Sistemleri ve Elektronik Bankacılık Hizmetleri Hakkında Yönetmelik (RG 15.03.2020) md. 25 — birincil ve ikincil sistemler yurt içinde</t>
         </is>
       </c>
-      <c r="S17" s="6" t="inlineStr">
+      <c r="T17" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T17" s="6" t="inlineStr">
+      <c r="U17" s="6" t="inlineStr">
         <is>
           <t>v0 "air-gap / activations cannot be exfiltrated" → gözlemlenebilir olan çıkış reddine indirgendi. Y-6: v0 L1 tanımı ("dış API yok") artık yalnız SOV profilinin kapısı.</t>
         </is>
       </c>
-      <c r="U17" s="6" t="inlineStr">
+      <c r="V17" s="6" t="inlineStr">
         <is>
           <t>Inference inside the governed boundary</t>
         </is>
       </c>
-      <c r="V17" s="6" t="inlineStr">
+      <c r="W17" s="6" t="inlineStr">
         <is>
           <t>All models run inside the boundary, egress is default deny with only listed internal destinations, and logs or a dated test show no other outbound connection.</t>
         </is>
@@ -2404,39 +2435,40 @@
           <t>2'yi karşılıyor; çağrı kayıtları 3 ay içinde G-SUP-01 ile karşılaştırılarak gözden geçiriliyor ve onaylı listeden çıkarılan bir sağlayıcının 5 iş günü içinde engellendiği kayıtla gösteriliyor.</t>
         </is>
       </c>
-      <c r="P18" s="6" t="n">
+      <c r="P18" s="6" t="inlineStr"/>
+      <c r="Q18" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Q18" s="6" t="inlineStr">
+      <c r="R18" s="6" t="inlineStr">
         <is>
           <t>[DOC] Onaylı sağlayıcılar, uç noktalar ve kurum hesapları listesi (G-SUP-01 ile tutarlı)
 [CFG] Yalnız listelenmiş hedeflere izin veren kontrollü nokta yapılandırması (gateway, proxy ya da çıkış kuralları)
 [LOG] Son 30 güne ait sağlayıcı, uç nokta, çağıran sistem ve zaman içeren çağrı kayıtları</t>
         </is>
       </c>
-      <c r="R18" s="6" t="inlineStr">
+      <c r="S18" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 9, md. 12(1)
 ISO/IEC 27001:2022 A.5.23, A.8.20
 ISO/IEC 42001 Annex A.10.3 (suppliers)</t>
         </is>
       </c>
-      <c r="S18" s="6" t="inlineStr">
+      <c r="T18" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-03, AS-04</t>
         </is>
       </c>
-      <c r="T18" s="6" t="inlineStr">
+      <c r="U18" s="6" t="inlineStr">
         <is>
           <t>Y-6'nın CE tarafı: SOV'un "dış çağrı yok" kapısının CE karşılığı "dış çağrı yalnız kontrollü noktadan". Kontrollü nokta tipik olarak AI gateway (Y-9 ile ilişkili); madde teknolojiden bağımsız yazıldı.</t>
         </is>
       </c>
-      <c r="U18" s="6" t="inlineStr">
+      <c r="V18" s="6" t="inlineStr">
         <is>
           <t>External inference only through sanctioned endpoints</t>
         </is>
       </c>
-      <c r="V18" s="6" t="inlineStr">
+      <c r="W18" s="6" t="inlineStr">
         <is>
           <t>Every system calls external models only through the controlled point, only sanctioned destinations and organisation accounts are reachable, direct egress to providers is blocked, and calls from the last 30 days are logged.</t>
         </is>
@@ -2510,17 +2542,18 @@
           <t>2'yi karşılıyor; kayıt 6 ay içinde çalışan yapılandırmayla karşılaştırılmış ve kaynak eklemek kayıtlı bir onay gerektiriyor.</t>
         </is>
       </c>
-      <c r="P19" s="6" t="n">
+      <c r="P19" s="6" t="inlineStr"/>
+      <c r="Q19" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q19" s="6" t="inlineStr">
+      <c r="R19" s="6" t="inlineStr">
         <is>
           <t>[DOC] Onaylı kaynak kaydı (kaynak, sahip, veri kategorileri, giriş yolu, onay tarihi)
 [CFG] Her giriş yolunda kabul edilen kaynakları sınırlayan yapılandırma (izin listesi, bağlayıcı kapsamı, yükleme yetkileri)
 [LOG] Onaysız kaynak ret kayıtları; son 90 günde olmadıysa test kaydı</t>
         </is>
       </c>
-      <c r="R19" s="6" t="inlineStr">
+      <c r="S19" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.8.20, A.5.14
 ISO/IEC 42001 Annex A.7.3 (acquisition of data)
@@ -2528,22 +2561,22 @@
 NIS2 Art. 21(2)</t>
         </is>
       </c>
-      <c r="S19" s="6" t="inlineStr">
+      <c r="T19" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T19" s="6" t="inlineStr">
+      <c r="U19" s="6" t="inlineStr">
         <is>
           <t>v0 "approved sources, formats and protocols" üç gereksinimi tek cümlede topluyordu; format/protokol doğrulaması BEH-ING'e (şema) gider. Kaynak kimlik doğrulaması IDE-ING-01.</t>
         </is>
       </c>
-      <c r="U19" s="6" t="inlineStr">
+      <c r="V19" s="6" t="inlineStr">
         <is>
           <t>Approved data sources only</t>
         </is>
       </c>
-      <c r="V19" s="6" t="inlineStr">
+      <c r="W19" s="6" t="inlineStr">
         <is>
           <t>Every source in use is in the register, every path accepts only registered sources, and rejection logs or a dated test record show an unapproved source being rejected.</t>
         </is>
@@ -2613,17 +2646,18 @@
           <t>2'yi karşılıyor; sertifika süreleri ve protokol yapılandırması alarmla izleniyor ve test 6 ay içinde tekrarlanıyor.</t>
         </is>
       </c>
-      <c r="P20" s="6" t="n">
+      <c r="P20" s="6" t="inlineStr"/>
+      <c r="Q20" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q20" s="6" t="inlineStr">
+      <c r="R20" s="6" t="inlineStr">
         <is>
           <t>[DOC] Akış başına protokolü gösteren veri akışları listesi (veri akış şemasından)
 [CFG] Uç noktalarda ve servisler arası bağlantılarda protokol ve asgari sürüm yapılandırması
 [TST] Son 6 ay içinde tarihli, şifresiz ya da eskimiş protokollü uç nokta olmadığını gösteren tarama/test sonucu</t>
         </is>
       </c>
-      <c r="R20" s="6" t="inlineStr">
+      <c r="S20" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 12(1)
 GDPR Art. 32(1)(a)
@@ -2631,22 +2665,22 @@
 NIS2 Art. 21(2)(h)</t>
         </is>
       </c>
-      <c r="S20" s="6" t="inlineStr">
+      <c r="T20" s="6" t="inlineStr">
         <is>
           <t>AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T20" s="6" t="inlineStr">
+      <c r="U20" s="6" t="inlineStr">
         <is>
           <t>v0 seviye metninde L0 şartıydı ama hücresi yoktu (01-hucre-analizi bulgu 2). CON-ING altında açıldı çünkü sınır kontrolü; tüm aşamaları kapsar. QS'de yok: beyanla cevap neredeyse her zaman "evet", bilgi değeri düşük.</t>
         </is>
       </c>
-      <c r="U20" s="6" t="inlineStr">
+      <c r="V20" s="6" t="inlineStr">
         <is>
           <t>Encryption in transit</t>
         </is>
       </c>
-      <c r="V20" s="6" t="inlineStr">
+      <c r="W20" s="6" t="inlineStr">
         <is>
           <t>Every flow in the list, internal and external, is encrypted, deprecated versions are refused, and a test result from the last 6 months confirms it.</t>
         </is>
@@ -2716,39 +2750,40 @@
           <t>2'yi karşılıyor; kurallar 6 ay içinde envanterle karşılaştırılmış ve kural değişiklikleri kayıtlı onay gerektiriyor.</t>
         </is>
       </c>
-      <c r="P21" s="6" t="n">
+      <c r="P21" s="6" t="inlineStr"/>
+      <c r="Q21" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q21" s="6" t="inlineStr">
+      <c r="R21" s="6" t="inlineStr">
         <is>
           <t>[DOC] Her depoya erişebilen bileşenleri gösteren depo envanteri
 [CFG] Varsayılan reddi ve izinli akışları gösteren ağ politikası ya da firewall kuralları
 [TST] İzinsiz bir bileşenden yapılmış, tarihli bağlantı testi</t>
         </is>
       </c>
-      <c r="R21" s="6" t="inlineStr">
+      <c r="S21" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.8.22
 KVKK md. 12(1)
 NIS2 Art. 21(2)</t>
         </is>
       </c>
-      <c r="S21" s="6" t="inlineStr">
+      <c r="T21" s="6" t="inlineStr">
         <is>
           <t>AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T21" s="6" t="inlineStr">
+      <c r="U21" s="6" t="inlineStr">
         <is>
           <t>Belge düzeyinde yetki (A kullanıcısı B'nin belgesi) burada değil, IDE-STO / IDE-INF'te. Bu madde ağ düzeyi.</t>
         </is>
       </c>
-      <c r="U21" s="6" t="inlineStr">
+      <c r="V21" s="6" t="inlineStr">
         <is>
           <t>Segmentation of AI data stores</t>
         </is>
       </c>
-      <c r="V21" s="6" t="inlineStr">
+      <c r="W21" s="6" t="inlineStr">
         <is>
           <t>Every store in the inventory is segmented with default deny, allowed flows match the inventory, and a dated test shows a non-allowed component is refused.</t>
         </is>
@@ -2822,39 +2857,40 @@
           <t>2'yi karşılıyor ve anahtar rotasyonu ya da anahtarlara erişim 12 ay içinde gözden geçirilmiş, kaydı var.</t>
         </is>
       </c>
-      <c r="P22" s="6" t="n">
+      <c r="P22" s="6" t="inlineStr"/>
+      <c r="Q22" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q22" s="6" t="inlineStr">
+      <c r="R22" s="6" t="inlineStr">
         <is>
           <t>[DOC] Depo başına şifreleme durumu ve anahtar sahibini gösteren depo envanteri (CON-STO-01 + sağlayıcı depoları ve yedekler)
 [CFG] Kurumun işlettiği depolar için şifreleme yapılandırması
 [DOC] Sağlayıcının işlettiği depolar için sağlayıcı belgeleri</t>
         </is>
       </c>
-      <c r="R22" s="6" t="inlineStr">
+      <c r="S22" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 12(1)
 GDPR Art. 32(1)(a)
 ISO/IEC 27001:2022 A.8.24</t>
         </is>
       </c>
-      <c r="S22" s="6" t="inlineStr">
+      <c r="T22" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02</t>
         </is>
       </c>
-      <c r="T22" s="6" t="inlineStr">
+      <c r="U22" s="6" t="inlineStr">
         <is>
           <t>v0'da hücresi olmayan L1 şartı. Anahtar sahibi bilgisi SOV iddiası için G-SUP-02'ye girdi. Kayıt ve yedeklerin açıkça sayılması bilinçli: tipik açık orada.</t>
         </is>
       </c>
-      <c r="U22" s="6" t="inlineStr">
+      <c r="V22" s="6" t="inlineStr">
         <is>
           <t>Encryption at rest with controlled keys</t>
         </is>
       </c>
-      <c r="V22" s="6" t="inlineStr">
+      <c r="W22" s="6" t="inlineStr">
         <is>
           <t>Every store in the inventory, including logs, indexes and backups, is encrypted at rest with configuration or provider evidence, and the key holder is recorded for each.</t>
         </is>
@@ -2928,17 +2964,18 @@
           <t>2'yi karşılıyor ve liste 12 ay içinde ya da son veri kaynağı eklendikten sonra (hangisi önce gelirse) gözden geçirilmiş; tarihli gözden geçirme kaydı var.</t>
         </is>
       </c>
-      <c r="P23" s="6" t="n">
+      <c r="P23" s="6" t="inlineStr"/>
+      <c r="Q23" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q23" s="6" t="inlineStr">
+      <c r="R23" s="6" t="inlineStr">
         <is>
           <t>[DOC] Veri kaynağı başına kategori listesi (ör. TCKN, IBAN, kart numarası, telefon, adres, sağlık verisi)
 [DOC] Muamele tablosu: kategori -&gt; engelle / maskele / takma adlandır / izin ver; 'izin ver' için dayanak
 [DOC] Sahibini adıyla gösteren onay kaydı</t>
         </is>
       </c>
-      <c r="R23" s="6" t="inlineStr">
+      <c r="S23" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 4(2)(ç)
 KVKK md. 6
@@ -2947,22 +2984,22 @@
 ISO/IEC 42001 Annex A.7.2, A.7.6 (data for development; data preparation)</t>
         </is>
       </c>
-      <c r="S23" s="6" t="inlineStr">
+      <c r="T23" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-07</t>
         </is>
       </c>
-      <c r="T23" s="6" t="inlineStr">
+      <c r="U23" s="6" t="inlineStr">
         <is>
           <t>HYG-ING-02..04 ve HYG-RES için ön koşul: hedef tanımlanmadan tespit ölçülemez. AS-07 veri haritasına da girdi.</t>
         </is>
       </c>
-      <c r="U23" s="6" t="inlineStr">
+      <c r="V23" s="6" t="inlineStr">
         <is>
           <t>Personal data scope and treatment defined</t>
         </is>
       </c>
-      <c r="V23" s="6" t="inlineStr">
+      <c r="W23" s="6" t="inlineStr">
         <is>
           <t>The list covers every in-scope data source, includes special categories and the relevant locale-specific identifiers, defines a treatment per category, and is approved by a named owner.</t>
         </is>
@@ -3018,35 +3055,47 @@
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>Hiçbir giriş yolunda otomatik tespit yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: kontrol yolların yalnız bir kısmında; tespit edip kaydediyor ama muameleyi uygulamıyor; veri saklandıktan ya da indekslendikten sonra çalışıyor; muamele elle yapılıyor; kayıt kanıtı sunulamıyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>Envanterdeki her yolda kontrol saklama/indeksleme öncesinde var, HYG-ING-01'deki muamele uygulanıyor ve son 30 günde veri alan her yol için o döneme ait kayıt var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; değişiklik yönetiminde hiçbir yeni giriş yolunun kontrol olmadan canlıya alınmadığını güvenceye alan bir kontrol adımı var; yol envanteri 6 ay içinde çalışan sistemle karşılaştırılmış, tarihli kaydı var.</t>
-        </is>
-      </c>
-      <c r="P24" s="6" t="n">
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P24" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir veri giriş yolunda kişisel veriyi otomatik tespit eden bir kontrol var.
+c2 [temel] Giriş yolu envanteri var.
+c3 [temel] Envanterdeki yollardan tespit kontrolü bulunanların oranı. [%100 (hepsi)]
+c4 [temel] Kontrol bulunan yollardan kontrolün saklamadan önce çalıştığı yolların oranı. [%100 (hepsi)]
+c5 [temel] Kontrol HYG-ING-01'deki muameleyi otomatik uyguluyor (yalnız kaydetmiyor, elle adım gerekmiyor).
+c6 [temel, QS dışı] Son 30 günde veri alan yollardan, o döneme ait tespit/muamele kaydı bulunanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Değişiklik sürecinde, yeni bir giriş yolunun kontrol olmadan canlıya alınmasını engelleyen bir adım var.
+s2 [sürdürme] Yol envanteri çalışan sistemle karşılaştırılmış; tarihli kaydı 6 ay içinde. [≤ 6 ay]</t>
+        </is>
+      </c>
+      <c r="Q24" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q24" s="6" t="inlineStr">
+      <c r="R24" s="6" t="inlineStr">
         <is>
           <t>[DOC] Veri giriş yolları envanteri (mimari ya da veri akış şeması)
 [CFG] Kontrolün her yoldaki varlığını ve saklama/indeksleme öncesindeki yerini gösteren yapılandırma
 [LOG] Son 30 güne ait, her yoldan tespit/muamele kayıtları</t>
         </is>
       </c>
-      <c r="R24" s="6" t="inlineStr">
+      <c r="S24" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 12(1)
 GDPR Art. 25(1)
@@ -3054,24 +3103,24 @@
 ISO/IEC 27001:2022 A.8.11</t>
         </is>
       </c>
-      <c r="S24" s="6" t="inlineStr">
+      <c r="T24" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T24" s="6" t="inlineStr">
+      <c r="U24" s="6" t="inlineStr">
         <is>
           <t>v0'daki "every ingested data item" yerine "every in-scope path": yol gözlemlenebilir, tek tek öğe gözlemlenemez. Araç seçenekleri: tool reference (HYG-ING).</t>
         </is>
       </c>
-      <c r="U24" s="6" t="inlineStr">
+      <c r="V24" s="6" t="inlineStr">
         <is>
           <t>Automated detection and treatment before persistence</t>
         </is>
       </c>
-      <c r="V24" s="6" t="inlineStr">
-        <is>
-          <t>Every path in the inventory has the control before storage/indexing, the treatment from HYG-ING-01 is applied, and log events from the last 30 days exist for every path that received data in that period.</t>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -3139,39 +3188,40 @@
           <t>2'yi karşılıyor; test, tespit bileşeninin her değişikliğinde ve en geç 6 ay içinde tekrarlanıyor; karantina olayları alarm üretiyor ve alarmın ele alındığına dair kayıt var.</t>
         </is>
       </c>
-      <c r="P25" s="6" t="n">
+      <c r="P25" s="6" t="inlineStr"/>
+      <c r="Q25" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q25" s="6" t="inlineStr">
+      <c r="R25" s="6" t="inlineStr">
         <is>
           <t>[CFG] Her yolda hata/zaman aşımı davranışını gösteren yapılandırma
 [TST] Tarihli test kaydı: kontrol durduruldu, desteklenmeyen girdi gönderildi, sonuç gözlendi
 [LOG] Karantina/ret kayıtları</t>
         </is>
       </c>
-      <c r="R25" s="6" t="inlineStr">
+      <c r="S25" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 12(1)
 GDPR Art. 32(1)(b)
 ISO/IEC 27001:2022 A.8.11</t>
         </is>
       </c>
-      <c r="S25" s="6" t="inlineStr">
+      <c r="T25" s="6" t="inlineStr">
         <is>
           <t>AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T25" s="6" t="inlineStr">
+      <c r="U25" s="6" t="inlineStr">
         <is>
           <t>v0'da yalnız stack guide'da araç notuydu. Fail-open bir tespit bileşeni HYG-ING-02'yi anlamsız kıldığı için maddeye yükseltildi. Quick Scan'de yok: müşteri test etmeden cevabı nadiren bilir.</t>
         </is>
       </c>
-      <c r="U25" s="6" t="inlineStr">
+      <c r="V25" s="6" t="inlineStr">
         <is>
           <t>Detection fails closed</t>
         </is>
       </c>
-      <c r="V25" s="6" t="inlineStr">
+      <c r="W25" s="6" t="inlineStr">
         <is>
           <t>Fail-closed is configured on every path for unavailability, error/timeout and unsupported language/format, and a dated test record shows data blocked or quarantined in each class.</t>
         </is>
@@ -3241,39 +3291,40 @@
           <t>2'yi karşılıyor; ölçüm tespit yapılandırmasının ya da modelinin her değişikliğinde ve en geç 6 ay içinde tekrarlanıyor; sonuçlar zaman serisi olarak saklanıyor.</t>
         </is>
       </c>
-      <c r="P26" s="6" t="n">
+      <c r="P26" s="6" t="inlineStr"/>
+      <c r="Q26" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q26" s="6" t="inlineStr">
+      <c r="R26" s="6" t="inlineStr">
         <is>
           <t>[DOC] Bilinen-cevaplı test setinin tanımı (sentetik), kategoriler ve adetler
 [TST] Kategori başına tespit oranı (recall) sonucu, tarihli
 [DOC] Sahibin belirlediği kategori başına eşik; eşiğin altındaki kategoriler için aksiyon kaydı</t>
         </is>
       </c>
-      <c r="R26" s="6" t="inlineStr">
+      <c r="S26" s="6" t="inlineStr">
         <is>
           <t>GDPR Art. 32(1)(d)
 NIST AI RMF MEASURE 2.10 (privacy risk examined and documented)
 ISO/IEC 42001 Annex A.6.2.4 (verification and validation)</t>
         </is>
       </c>
-      <c r="S26" s="6" t="inlineStr">
+      <c r="T26" s="6" t="inlineStr">
         <is>
           <t>AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T26" s="6" t="inlineStr">
+      <c r="U26" s="6" t="inlineStr">
         <is>
           <t>L1 değil L3: L1 kontrolün var olmasını ve fail-closed çalışmasını ister; L3 kalitesinin bilinmesini. Tipik açık Türkçe kapsamı.</t>
         </is>
       </c>
-      <c r="U26" s="6" t="inlineStr">
+      <c r="V26" s="6" t="inlineStr">
         <is>
           <t>Detection effectiveness measured</t>
         </is>
       </c>
-      <c r="V26" s="6" t="inlineStr">
+      <c r="W26" s="6" t="inlineStr">
         <is>
           <t>Measured with a known-answer set covering every category in HYG-ING-01; per-category recall recorded; each category meets its threshold or has an open action with owner and date.</t>
         </is>
@@ -3347,39 +3398,40 @@
           <t>2'yi karşılıyor; atlatmalar ve tespitler 3 ay içinde gözden geçiriliyor, aksiyonlar kayıtlı.</t>
         </is>
       </c>
-      <c r="P27" s="6" t="n">
+      <c r="P27" s="6" t="inlineStr"/>
+      <c r="Q27" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Q27" s="6" t="inlineStr">
+      <c r="R27" s="6" t="inlineStr">
         <is>
           <t>[DOC] Prompt'lar için kategori ve muamele listesi (HYG-ING-01 kullanılabilir; serbest metin ve ekleri kapsamalı)
 [CFG] Kontrolün her prompt kanalında (arayüz, API, eklentiler) model çağrısından önce bulunduğunu gösteren yapılandırma
 [LOG] Kanal başına son 30 güne ait tespit/muamele kayıtları</t>
         </is>
       </c>
-      <c r="R27" s="6" t="inlineStr">
+      <c r="S27" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 9, md. 12(1)
 GDPR Art. 25(1), Art. 32(1)(a)
 ISO/IEC 27001:2022 A.8.11, A.8.12</t>
         </is>
       </c>
-      <c r="S27" s="6" t="inlineStr">
+      <c r="T27" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-03, AS-07</t>
         </is>
       </c>
-      <c r="T27" s="6" t="inlineStr">
+      <c r="U27" s="6" t="inlineStr">
         <is>
           <t>v0 HYG-PRM'nin PII yarısı; injection yarısı BEH-PRM'e gidiyor (01-hucre-analizi). CE'de L1: verinin kurumdan çıktığı nokta. Fail-closed ve etkinlik maddeleri (HYG-PRM-02/03) HYG-ING-03/04 kalıbıyla matris oturumlarında yazılacak.</t>
         </is>
       </c>
-      <c r="U27" s="6" t="inlineStr">
+      <c r="V27" s="6" t="inlineStr">
         <is>
           <t>Personal data in prompts treated before the model</t>
         </is>
       </c>
-      <c r="V27" s="6" t="inlineStr">
+      <c r="W27" s="6" t="inlineStr">
         <is>
           <t>Every prompt channel, including attachments, applies the defined treatment before the model call; any user override requires a logged reason; events from the last 30 days exist for every channel used in that period.</t>
         </is>
@@ -3449,39 +3501,40 @@
           <t>2'yi karşılıyor; kaynak kimlik bilgileri 6 ay içinde gözden geçirilmiş ve kullanılmayanlar iptal edilmiş, kaydı var.</t>
         </is>
       </c>
-      <c r="P28" s="6" t="n">
+      <c r="P28" s="6" t="inlineStr"/>
+      <c r="Q28" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q28" s="6" t="inlineStr">
+      <c r="R28" s="6" t="inlineStr">
         <is>
           <t>[CFG] Giriş yolu başına kimlik doğrulama yapılandırması (servis kimlik bilgileri, yüklemeler için kullanıcı girişi)
 [DOC] Paylaşımlı ya da anonim kimlik bilgisi olmadığını gösteren kaynak başına kimlik bilgisi listesi
 [TST] Kimliği doğrulanmamış bir gönderimin reddedildiğini gösteren tarihli test</t>
         </is>
       </c>
-      <c r="R28" s="6" t="inlineStr">
+      <c r="S28" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.5.16, A.5.17, A.8.5
 KVKK md. 12(1)
 SOC 2 CC6.1</t>
         </is>
       </c>
-      <c r="S28" s="6" t="inlineStr">
+      <c r="T28" s="6" t="inlineStr">
         <is>
           <t>AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T28" s="6" t="inlineStr">
+      <c r="U28" s="6" t="inlineStr">
         <is>
           <t>v0'daki "provenance is logged" TRA-ING-01'e taşındı. QS'de yok: CON-ING-01 aynı riski beyan düzeyinde yeterince yakalıyor.</t>
         </is>
       </c>
-      <c r="U28" s="6" t="inlineStr">
+      <c r="V28" s="6" t="inlineStr">
         <is>
           <t>Authenticated sources</t>
         </is>
       </c>
-      <c r="V28" s="6" t="inlineStr">
+      <c r="W28" s="6" t="inlineStr">
         <is>
           <t>Every path requires authentication with individual credentials, credentials expire or rotate on a defined period, and a dated test shows rejection of an unauthenticated submission.</t>
         </is>
@@ -3555,39 +3608,40 @@
           <t>2'yi karşılıyor; erişim gözden geçirmeleri 6 ay içinde yapılıyor ve ayrılan çalışanların erişiminin 2 iş günü içinde kaldırıldığı kayıtlarla gösteriliyor.</t>
         </is>
       </c>
-      <c r="P29" s="6" t="n">
+      <c r="P29" s="6" t="inlineStr"/>
+      <c r="Q29" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Q29" s="6" t="inlineStr">
+      <c r="R29" s="6" t="inlineStr">
         <is>
           <t>[DOC] Her depo için rol tanımları ve rol başına kimlik listesi
 [CFG] Her depo için erişim kontrol yapılandırması (ya da yetki dökümü)
 [DOC] Tarih, gözden geçiren ve kaldırılan erişimleri içeren erişim gözden geçirme kaydı</t>
         </is>
       </c>
-      <c r="R29" s="6" t="inlineStr">
+      <c r="S29" s="6" t="inlineStr">
         <is>
           <t>KVKK md. 12(1)
 ISO/IEC 27001:2022 A.5.15, A.5.18, A.8.3
 GDPR Art. 32(1)(b)</t>
         </is>
       </c>
-      <c r="S29" s="6" t="inlineStr">
+      <c r="T29" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AS-03</t>
         </is>
       </c>
-      <c r="T29" s="6" t="inlineStr">
+      <c r="U29" s="6" t="inlineStr">
         <is>
           <t>Prompt/yanıt kayıtları açıkça sayıldı: çoğu kurumda en hassas ve en az korunan depo. Secret yönetimi (v0 seviye metni) ayrı madde olarak IDE-STO-02'de yazılacak (oturum 4+). Model üzerinden belge yetkisi (RAG) IDE-INF'te.</t>
         </is>
       </c>
-      <c r="U29" s="6" t="inlineStr">
+      <c r="V29" s="6" t="inlineStr">
         <is>
           <t>Role-based access to AI data and artefacts</t>
         </is>
       </c>
-      <c r="V29" s="6" t="inlineStr">
+      <c r="W29" s="6" t="inlineStr">
         <is>
           <t>Every store, including prompt and response logs, has defined roles, only named identities hold access, permissions match the role definitions, and an access review was done in the last 12 months.</t>
         </is>
@@ -3661,17 +3715,18 @@
           <t>2'yi karşılıyor; kayıt bütünlüğü 3 ay içinde doğrulanıyor (ör. özet kontrolü ya da boşluk tespiti) ve kaydı var; kayıt saklama süresi tanımlı süreyle örtüşüyor.</t>
         </is>
       </c>
-      <c r="P30" s="6" t="n">
+      <c r="P30" s="6" t="inlineStr"/>
+      <c r="Q30" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Q30" s="6" t="inlineStr">
+      <c r="R30" s="6" t="inlineStr">
         <is>
           <t>[CFG] Her giriş yolunda dört alanı (kaynak, zaman, kategoriler, muamele) içeren kayıt yapılandırması
 [CFG] Kayıt deposu koruması (yalnız ekleme ya da tek yazım ayarı, sistem yöneticilerinden ayrı yetki ya da bütünlük doğrulaması)
 [TST] Saklanan üç örnek öğenin kayıt girdilerine kadar izlenmesi</t>
         </is>
       </c>
-      <c r="R30" s="6" t="inlineStr">
+      <c r="S30" s="6" t="inlineStr">
         <is>
           <t>ISO/IEC 27001:2022 A.8.15
 ISO/IEC 42001 Annex A.7.5
@@ -3679,29 +3734,29 @@
 KVKK md. 12(1)</t>
         </is>
       </c>
-      <c r="S30" s="6" t="inlineStr">
+      <c r="T30" s="6" t="inlineStr">
         <is>
           <t>AS-01, AS-02, AU-01</t>
         </is>
       </c>
-      <c r="T30" s="6" t="inlineStr">
+      <c r="U30" s="6" t="inlineStr">
         <is>
           <t>v0 "immutable and tamper-evident" ölçütsüzdü; üç mekanizmadan biri şartı ölçülebilir kıldı. Tek başına "log tutuluyor" 1 puan.</t>
         </is>
       </c>
-      <c r="U30" s="6" t="inlineStr">
+      <c r="V30" s="6" t="inlineStr">
         <is>
           <t>Tamper-evident provenance log</t>
         </is>
       </c>
-      <c r="V30" s="6" t="inlineStr">
+      <c r="W30" s="6" t="inlineStr">
         <is>
           <t>Every path logs the four fields, the log store is protected by at least one of the listed mechanisms, and all three sampled items are traced to their entries.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V30"/>
+  <autoFilter ref="A1:W30"/>
   <dataValidations count="1">
     <dataValidation sqref="B2:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Onay,Düzelt,Sil,Tartışalım"</formula1>

</xml_diff>

<commit_message>
A2 adım 3: kalan 16 QS maddesi kontrol listesine çevrildi
- 16 madde (G 9, CON 4, HYG 2, IDE 1, TRA 1) checks ile; elle yazılmış rubric kaldırıldı
- QS kesitinde 18 madde, 120 kontrol; terms.yaml 33 terim
- rehber/CSV/tablo/xlsx yeniden üretildi; schema 5.5, README, meta changelog

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RaFMgY52inRvN44BSaYeeZ
</commit_message>
<xml_diff>
--- a/measurement-tool/output/inceleme-paketi.xlsx
+++ b/measurement-tool/output/inceleme-paketi.xlsx
@@ -724,25 +724,36 @@
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>AI olayları hiçbir prosedürde ele alınmıyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M2" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: prosedür dört AI olay türünü adlandırmıyor; raporlama zincirinde adı belli roller yok; uygulanan bildirim süreleri eksik; genel olay süreciyle bağlantılı değil.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N2" s="6" t="inlineStr">
         <is>
-          <t>Prosedür dört olay türünü, adı belli rollerle raporlama zincirini ve uygulanan süreleri tanımlıyor, genel süreçle bağlantılı ve son 12 ayda bir tatbikat ya da ele alınmış bir AI olayı kayıtlı.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O2" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; her tatbikat ya da olaydan çıkan dersler kayıtlı, aksiyonlar kapanışa kadar izleniyor ve prosedür 12 ay içinde gözden geçirilmiş.</t>
-        </is>
-      </c>
-      <c r="P2" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] AI olayları bir olay prosedüründe ele alınıyor (ayrı ya da genel prosedürün içinde).
+c2 [temel] Prosedür dört AI olay türünün hepsini adlandırıyor.
+c3 [temel] Raporlama zinciri adı belli rollerle tanımlı.
+c4 [temel] Uygulanan bildirim sürelerinin tablosu var.
+c5 [temel, QS dışı] Prosedür genel güvenlik olay süreciyle bağlantılı (ortak giriş noktası ya da açık devir adımı).
+c6 [temel] Son tatbikatın ya da ele alınmış AI olayı kaydının tarihi son 12 ay içinde. [≤ 12 ay]
+s1 [sürdürme] Her tatbikat ya da olaydan çıkan dersler kayıtlı ve aksiyonlar kapanışa kadar izleniyor.
+s2 [sürdürme] Prosedür gözden geçirilmiş; tarihli kaydı 12 ay içinde. [≤ 12 ay]</t>
+        </is>
+      </c>
       <c r="Q2" s="6" t="n">
         <v>12</v>
       </c>
@@ -780,7 +791,7 @@
       </c>
       <c r="W2" s="6" t="inlineStr">
         <is>
-          <t>The procedure names the four incident types, the reporting chain with named roles and the applicable deadlines, is linked to the general process, and an exercise or a handled AI incident is recorded in the last 12 months.</t>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -834,25 +845,33 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>AI sistemleri ya da kullanım senaryoları için envanter yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>Envanter var ama şunlardan en az biri geçerli: bir ya da daha fazla kayıtta zorunlu bir alan boş; satın alma kayıtlarında, onaylı araç listesinde ya da görüşmelerde görülen bir sistem envanterde yok; son 6 ayda güncellenmemiş.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c4) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>Her kayıtta tüm zorunlu alanlar dolu; satın alma kayıtlarında, onaylı araç listesinde ya da görüşmelerde görülen hiçbir sistem eksik değil; envanter son 6 ayda güncellenmiş.</t>
+          <t>c1 ve tüm temel kontroller (c2–c4) karşılanıyor.</t>
         </is>
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve envanter 6 ay içinde G-INV-02 trafik verileriyle karşılaştırılmış; eklenen ve çıkarılan kayıtların tarihli kaydı var.</t>
-        </is>
-      </c>
-      <c r="P3" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] AI sistemleri ve kullanım senaryoları envanteri var.
+c2 [temel] Envanter kayıtlarından tüm zorunlu alanları dolu olanların oranı. [%100 (hepsi)]
+c3 [temel] Satın alma kayıtlarında, onaylı araç listesinde (G-POL-02) ya da görüşmelerde görülen sistemlerden envanterde bulunanların oranı. [%100 (hepsi)]
+c4 [temel] Envanterin son güncelleme tarihi son 6 ay içinde. [≤ 6 ay]
+s1 [sürdürme] Envanter G-INV-02 trafik verisiyle karşılaştırılmış, eklenen ve çıkarılan kayıtlar yazılmış; tarihli kaydı 6 ay içinde. [≤ 6 ay]</t>
+        </is>
+      </c>
       <c r="Q3" s="6" t="n">
         <v>6</v>
       </c>
@@ -888,7 +907,7 @@
       </c>
       <c r="W3" s="6" t="inlineStr">
         <is>
-          <t>Every entry has all required fields, no system found in procurement records, the sanctioned tool list or interviews is missing, and the inventory was updated in the last 6 months.</t>
+          <t>c1 and all core checks (c2–c4) met.</t>
         </is>
       </c>
     </row>
@@ -942,25 +961,35 @@
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>AI servislerine giden trafik tanımlanamıyor ya da ilgili kayıtlar tutulmuyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Kayıtlar var ama şunlardan en az biri geçerli: saklama 90 günden kısa; trafik bir birime ya da kullanıcı grubuna atfedilemiyor; AI servis alan adı listesi tutulmuyor; hiç rapor üretilmemiş.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>Kayıtlar en az 90 gün saklanıyor, trafik bir birime ya da kullanıcı grubuna atfedilebiliyor, AI servis alan adı listesi son 6 ayda güncellenmiş ve talep edildiğinde en az 30 günlük rapor üretilebiliyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; raporlar 3 ay içinde gözden geçiriliyor ve onaylı listede (G-POL-02) olmayan servislere giden trafik kayıtlı bir takip başlatıyor.</t>
-        </is>
-      </c>
-      <c r="P4" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Dış AI servislerine giden trafik DNS, proxy ya da firewall kayıtlarında tanımlanabiliyor.
+c2 [temel] Bu kayıtların saklama süresi (gün). [≥ 90]
+c3 [temel] Trafik bir birime ya da kullanıcı grubuna atfedilebiliyor.
+c4 [temel] AI servis alan adı listesinin son güncelleme tarihi son 6 ay içinde. [≤ 6 ay]
+c5 [temel] Talep edildiğinde birim bazında, en az 30 günü kapsayan rapor üretilebiliyor.
+s1 [sürdürme] Raporlar gözden geçirilmiş; tarihli kaydı 3 ay içinde. [≤ 3 ay]
+s2 [sürdürme] Onaylı listede (G-POL-02) olmayan bir servise giden trafik kayıtlı bir takip başlatıyor.</t>
+        </is>
+      </c>
       <c r="Q4" s="6" t="n">
         <v>3</v>
       </c>
@@ -994,7 +1023,7 @@
       </c>
       <c r="W4" s="6" t="inlineStr">
         <is>
-          <t>Logs are retained for at least 90 days, traffic is attributable to a unit or user group, the AI service domain list was updated in the last 6 months, and a report covering at least 30 days can be produced on request.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -1048,25 +1077,35 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Yapay zekâ okuryazarlık programı yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>Program var ama şunlardan en az biri geçerli: üç konudan birini atlıyor; tamamlama kaydedilmiyor; kayıtlı tamamlama AI kullanıcılarının %80'inin altında.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>Program üç konuyu kapsıyor ve AI kullanıcılarının en az %80'inin kayıtlı tamamlaması var; yeni kullanıcılar erişimden sonraki 60 gün içinde tamamlıyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; içerik 12 ay içinde güncellenmiş ve anlama ölçülüyor (sınav ya da uygulama), sonuçlar kayıtlı.</t>
-        </is>
-      </c>
-      <c r="P5" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Yapay zekâ okuryazarlık programı var.
+c2 [temel] Program içeriği üç konuyu kapsıyor.
+c3 [temel] Tamamlama kişi başına tarihli kayıt altında.
+c4 [temel] AI kullanıcılarından kayıtlı tamamlaması olanların oranı. [en az %80]
+c5 [temel, QS dışı] Son 12 ayda erişim alan kullanıcılardan erişimden sonraki 60 gün içinde tamamlayanların oranı. [%100 (hepsi)]
+s1 [sürdürme] İçeriğin son güncelleme tarihi 12 ay içinde. [≤ 12 ay]
+s2 [sürdürme] Anlama ölçülüyor (sınav ya da uygulama) ve sonuçlar kayıtlı.</t>
+        </is>
+      </c>
       <c r="Q5" s="6" t="n">
         <v>12</v>
       </c>
@@ -1101,7 +1140,7 @@
       </c>
       <c r="W5" s="6" t="inlineStr">
         <is>
-          <t>The programme covers the three topics and at least 80% of AI users have a recorded completion; new users complete it within 60 days of access.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -1358,25 +1397,35 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>Yapay zekâ politikası yok ve AI başka hiçbir onaylı politikada ele alınmıyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>Politika ya da taslak var ama şunlardan en az biri geçerli: üst yönetim ya da yetkilendirdiği bir kurul tarafından onaylanmamış; hesap verecek rolü belirtmiyor; yeni bir AI sisteminin nasıl onaylanacağını tanımlamıyor; çalışanlara duyurulduğuna dair kayıt yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>Politika üst yönetim ya da yetkilendirilmiş kurul tarafından onaylanmış, hesap verecek rolü belirtiyor, yeni AI sistemleri için onay yolunu tanımlıyor, G-POL-02'ye atıf yapıyor ve kapsamdaki tüm çalışanlara duyurulduğuna dair kayıt var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve politika 12 ay içinde gözden geçirilmiş; değişiklikleri ya da değişiklik olmadığını belirten tarihli kayıt var.</t>
-        </is>
-      </c>
-      <c r="P8" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P8" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Yazılı bir yapay zekâ politikası var ya da AI onaylı başka bir politikada ele alınıyor.
+c2 [temel] Politika üst yönetim ya da yetkilendirdiği bir kurul tarafından onaylanmış, onay kaydı var.
+c3 [temel] Politika hesap verecek rolü adlandırıyor.
+c4 [temel] Politika yeni bir AI sisteminin onay yolunu tanımlıyor.
+c5 [temel, QS dışı] Politika kabul edilebilir kullanım kurallarına (G-POL-02) atıf yapıyor.
+c6 [temel] Kapsamdaki tüm çalışanlara duyuru kaydı var.
+s1 [sürdürme] Politika gözden geçirilmiş; tarihli kaydı (değişiklikler ya da "değişiklik yok") 12 ay içinde. [≤ 12 ay]</t>
+        </is>
+      </c>
       <c r="Q8" s="6" t="n">
         <v>12</v>
       </c>
@@ -1411,7 +1460,7 @@
       </c>
       <c r="W8" s="6" t="inlineStr">
         <is>
-          <t>The policy is approved by top management or a delegated body, names the accountable role, defines the approval route for new AI systems, references G-POL-02, and a record shows it was communicated to all staff in scope.</t>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -1581,25 +1630,34 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>Adı belli sahip yok, yönetişim rolü yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: envanterdeki bir ya da daha fazla sistemin adı belli sahibi yok; yönetişim rolü resmî olarak atanmamış; DPO ve güvenlik için danışma noktaları tanımlı değil.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>Envanterdeki her sistemin adı belli sahibi var, yönetişim rolü resmî olarak atanmış, danışma noktaları tanımlı ve en az bir danışmanın yapıldığına dair kayıt var (ya da son 12 ayda tetiklenmediği belirtilmiş).</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve sahipler ile rol atamaları 12 ay içinde teyit edilmiş; personel değişikliği sonrası güncellemeleri de içeren tarihli kayıt var.</t>
-        </is>
-      </c>
-      <c r="P10" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P10" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir AI sisteminin adı belli sahibi var ya da bir AI yönetişim rolü atanmış.
+c2 [temel] Envanterdeki (G-INV-01) sistemlerden adı belli sahibi olanların oranı. [%100 (hepsi)]
+c3 [temel] AI yönetişim rolü resmî olarak atanmış (atama yazısı ya da görev tanımı).
+c4 [temel] DPO ve güvenlik için danışma noktaları tanımlı.
+c5 [temel, QS dışı] Son 12 ayda en az bir danışma kayıtlı ya da hiç tetiklenmediği kayıtla belirtilmiş.
+s1 [sürdürme] Sahipler ve rol atamaları, personel değişikliği sonrası güncellemeler dahil teyit edilmiş; tarihli kaydı 12 ay içinde. [≤ 12 ay]</t>
+        </is>
+      </c>
       <c r="Q10" s="6" t="n">
         <v>12</v>
       </c>
@@ -1631,7 +1689,7 @@
       </c>
       <c r="W10" s="6" t="inlineStr">
         <is>
-          <t>Every inventoried system has a named owner, the governance role is formally assigned, consultation points are defined, and at least one record shows a consultation took place (or none was triggered in the last 12 months, stated).</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -1685,25 +1743,35 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>Hiçbir AI sistemi için risk değerlendirmesi yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: yalnız bazı sistemler için değerlendirme var; yazılı yöntem yok; değerlendirmeler AI'ye özgü riskleri (prompt ile veri çıkışı, yanlış ya da zararlı çıktı, model üzerinden yetkisiz erişim, sağlayıcı bağımlılığı) ele almıyor; yeniden değerlendirme tetikleyicileri tanımlı değil.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>Canlıdaki her sistem için, yazılı yöntemle yapılmış, dört AI'ye özgü risk grubunu ele alan, muamele kararları sahip tarafından onaylanmış tarihli bir değerlendirme var ve yeniden değerlendirme tetikleyicileri tanımlı.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve her değerlendirme 12 ay içinde ya da her tetikleyici olaydan sonra (hangisi önce gelirse) tekrarlanmış, kayıtları var.</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir AI sistemi için yazılı risk değerlendirmesi var.
+c2 [temel] Kriterleri, ölçekleri ve kabul kuralını içeren yazılı bir risk değerlendirme yöntemi var.
+c3 [temel] Canlıdaki AI sistemlerinden bu yöntemle yapılmış tarihli yazılı risk değerlendirmesi olanların oranı. [%100 (hepsi)]
+c4 [temel] Değerlendirmelerden dört AI'ye özgü risk grubunun hepsini ele alanların oranı. [%100 (hepsi)]
+c5 [temel, QS dışı] Değerlendirmelerden muamele kararları sistem sahibince onaylanmış olanların oranı. [%100 (hepsi)]
+c6 [temel] Yeniden değerlendirme tetikleyicileri tanımlı.
+s1 [sürdürme] Değerlendirmelerden 12 ay içinde ve her tetikleyici olaydan sonra (hangisi önce gelirse) tekrarlanmış olanların oranı. [%100 (hepsi)]</t>
+        </is>
+      </c>
       <c r="Q11" s="6" t="n">
         <v>12</v>
       </c>
@@ -1739,7 +1807,7 @@
       </c>
       <c r="W11" s="6" t="inlineStr">
         <is>
-          <t>Every production system has a dated assessment made with the written method that addresses the four AI-specific risk groups, with treatment decisions signed off by the owner, and re-assessment triggers are defined.</t>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -1996,25 +2064,34 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>Dış AI servisleri hiçbir sağlayıcı değerlendirmesi olmadan kullanılıyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: yalnız bazı sağlayıcılar değerlendirilmiş; bir değerlendirme beş konudan birini atlıyor; değerlendirme ilk kullanımdan sonra tarihli; dayanılan sağlayıcı belgeleri saklanmamış.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>Kurum verisiyle kullanılan her sağlayıcının, beş konunun hepsini kapsayan, ilk kullanımdan önce tarihli değerlendirmesi var ve dayanılan sağlayıcı belgeleri saklanıyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve her değerlendirme 12 ay içinde ve sağlayıcı koşullarında ya da alt işleyenlerde bildirilen her değişiklikten sonra tekrarlanmış, kayıtları var.</t>
-        </is>
-      </c>
-      <c r="P14" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P14" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Kurum verisiyle kullanılan en az bir dış AI sağlayıcısı için yazılı değerlendirme var.
+c2 [temel] Kurum verisiyle kullanılan dış AI sağlayıcılarından yazılı değerlendirmesi olanların oranı. [%100 (hepsi)]
+c3 [temel] Değerlendirmelerden beş konunun hepsini kapsayanların oranı. [%100 (hepsi)]
+c4 [temel] Değerlendirmelerden kurum verisiyle ilk kullanımdan önce tarihli olanların oranı. [%100 (hepsi)]
+c5 [temel, QS dışı] Dayanılan sağlayıcı belgeleri (koşullar, veri işleme eki, alt işleyen listesi, veri yerleşimi beyanı) saklanıyor.
+s1 [sürdürme] Değerlendirmelerden 12 ay içinde ve sağlayıcı koşullarında ya da alt işleyenlerde bildirilen her değişiklikten sonra tekrarlanmış olanların oranı. [%100 (hepsi)]</t>
+        </is>
+      </c>
       <c r="Q14" s="6" t="n">
         <v>12</v>
       </c>
@@ -2050,7 +2127,7 @@
       </c>
       <c r="W14" s="6" t="inlineStr">
         <is>
-          <t>Every provider used with organisational data has an assessment covering all five topics, dated before first use, with the provider documents relied on retained.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -2310,25 +2387,35 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>Çıkarım ortamının dışarıya kısıtsız erişimi var ya da modeller dış bir servis üzerinden çağrılıyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>Modeller sınır içinde çalışıyor ama şunlardan en az biri geçerli: çıkış varsayılan red değil; listelenenler dışında dış hedefler var (ör. telemetri, çalışma anında model ya da paket indirme); kayıt ya da test kanıtı yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>Tüm modeller sınır içinde çalışıyor, çıkış yalnız listelenmiş iç hedeflerle varsayılan red ve kayıtlar ya da tarihli bir test başka bir dış bağlantı olmadığını gösteriyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; çıkarım ortamından dışarıya bağlantı denemeleri alarm üretiyor ve ele alınıyor; çıkış testi 6 ay içinde tekrarlanıyor.</t>
-        </is>
-      </c>
-      <c r="P17" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P17" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Sistemin en az bir modeli yönetilen sınır içinde çalışıyor (dış bir servis üzerinden değil).
+c2 [temel] Sistemin modellerinden yönetilen sınır içinde çalışanların oranı. [%100 (hepsi)]
+c3 [temel] Çıkarım ortamından çıkış varsayılan red; yalnız listelenmiş iç hedeflere izin var.
+c4 [temel] İzin listesinde hiçbir dış hedef yok (telemetri, çalışma anında model ya da paket indirme dahil).
+c5 [temel, QS dışı] En az 7 günlük çalışmaya ait çıkış/düşürme kayıtları ya da tarihli bir çıkış testi başka bir dış bağlantı olmadığını gösteriyor.
+s1 [sürdürme] Çıkarım ortamından dışarıya bağlantı denemesi alarm üretiyor ve her alarmın ele alınma kaydı var.
+s2 [sürdürme] Son çıkış testinin tarihi 6 ay içinde. [≤ 6 ay]</t>
+        </is>
+      </c>
       <c r="Q17" s="6" t="n">
         <v>6</v>
       </c>
@@ -2363,7 +2450,7 @@
       </c>
       <c r="W17" s="6" t="inlineStr">
         <is>
-          <t>All models run inside the boundary, egress is default deny with only listed internal destinations, and logs or a dated test show no other outbound connection.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -2417,25 +2504,36 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>Sistemler dış modelleri kontrollü nokta olmadan ya da kişisel hesap/anahtarla doğrudan çağırıyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>Kontrollü nokta var ama şunlardan en az biri geçerli: bazı sistemler onu atlıyor; hedefleri onaylı listeyle sınırlamıyor; kişisel hesap ya da anahtar kullanılıyor; çağrılar kaydedilmiyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>Her sistem dış modelleri yalnız kontrollü noktadan çağırıyor, yalnız onaylı hedeflere ve kurum hesaplarına erişilebiliyor, sağlayıcılara doğrudan çıkış engelli ve son 30 günün çağrıları kayıtlı.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; çağrı kayıtları 3 ay içinde G-SUP-01 ile karşılaştırılarak gözden geçiriliyor ve onaylı listeden çıkarılan bir sağlayıcının 5 iş günü içinde engellendiği kayıtla gösteriliyor.</t>
-        </is>
-      </c>
-      <c r="P18" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P18" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Dış model sağlayıcılarına yapılan çağrılar için kontrollü bir nokta var.
+c2 [temel] Controlled External sistemlerden dış modelleri yalnız kontrollü nokta üzerinden çağıranların oranı. [%100 (hepsi)]
+c3 [temel] Kontrollü nokta yalnız onaylı listedeki hedeflere ve kurum hesaplarına izin veriyor (G-SUP-01 ile tutarlı).
+c4 [temel] Kontrollü noktayı atlayarak sağlayıcı uç noktalarına doğrudan çıkış engelli.
+c5 [temel] Dış modelleri çağırmak için kişisel hesap ya da kişisel API anahtarı kullanılmıyor.
+c6 [temel] Son 30 günün çağrıları sağlayıcı, uç nokta, çağıran sistem ve zamanla kayıtlı.
+s1 [sürdürme] Çağrı kayıtları G-SUP-01 ile karşılaştırılarak gözden geçirilmiş; tarihli kaydı 3 ay içinde. [≤ 3 ay]
+s2 [sürdürme] Onaylı listeden çıkarılan her sağlayıcının kontrollü noktada 5 iş günü içinde engellendiği kayıtla gösteriliyor.</t>
+        </is>
+      </c>
       <c r="Q18" s="6" t="n">
         <v>3</v>
       </c>
@@ -2470,7 +2568,7 @@
       </c>
       <c r="W18" s="6" t="inlineStr">
         <is>
-          <t>Every system calls external models only through the controlled point, only sanctioned destinations and organisation accounts are reachable, direct egress to providers is blocked, and calls from the last 30 days are logged.</t>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -2524,25 +2622,34 @@
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>Kaynak kaydı yok ve giriş yollarında kısıt yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: kayıt var ama bir ya da daha fazla yol kayıt dışı kaynaklardan veri kabul ediyor; kısıt yapılandırılmış ama kayıt yok; ne ret kaydı ne test kaydı sunulabiliyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c4) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>Kullanılan her kaynak kayıtta, her yol yalnız kayıtlı kaynakları kabul ediyor ve ret kayıtları ya da tarihli bir test kaydı onaysız bir kaynağın reddedildiğini gösteriyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c4) karşılanıyor.</t>
         </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; kayıt 6 ay içinde çalışan yapılandırmayla karşılaştırılmış ve kaynak eklemek kayıtlı bir onay gerektiriyor.</t>
-        </is>
-      </c>
-      <c r="P19" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P19" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Sistem için onaylı veri kaynakları kaydı var.
+c2 [temel] Sistemi fiilen besleyen kaynaklardan kayıtta bulunanların oranı. [%100 (hepsi)]
+c3 [temel] Yalnız kayıtlı kaynaklardan veri kabul edecek biçimde yapılandırılmış giriş yollarının oranı. [%100 (hepsi)]
+c4 [temel, QS dışı] Onaysız bir kaynağın reddedildiğini gösteren son ret kaydının ya da tarihli testin tarihi. [≤ 90 gün]
+s1 [sürdürme] Kayıt çalışan yapılandırmayla karşılaştırılmış; tarihli kaydı 6 ay içinde. [≤ 6 ay]
+s2 [sürdürme] Kayda kaynak eklemek kayıtlı bir onay gerektiriyor.</t>
+        </is>
+      </c>
       <c r="Q19" s="6" t="n">
         <v>6</v>
       </c>
@@ -2578,7 +2685,7 @@
       </c>
       <c r="W19" s="6" t="inlineStr">
         <is>
-          <t>Every source in use is in the register, every path accepts only registered sources, and rejection logs or a dated test record show an unapproved source being rejected.</t>
+          <t>c1 and all core checks (c2–c4) met.</t>
         </is>
       </c>
     </row>
@@ -2839,25 +2946,33 @@
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Kişisel ya da gizli veri tutan bir ya da daha fazla depo şifresiz ya da durum bilinmiyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>Ana depolar şifreli ama şunlardan en az biri geçerli: kayıtlar, indeksler ya da yedekler şifresiz; her depo için anahtar sahibi belirlenmemiş; yapılandırma ya da sağlayıcı kanıtı sunulamıyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c4) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>Kayıtlar, indeksler ve yedekler dahil envanterdeki her depo depolamada şifreli, yapılandırma ya da sağlayıcı kanıtı var ve her biri için anahtar sahibi kayıtlı.</t>
+          <t>c1 ve tüm temel kontroller (c2–c4) karşılanıyor.</t>
         </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve anahtar rotasyonu ya da anahtarlara erişim 12 ay içinde gözden geçirilmiş, kaydı var.</t>
-        </is>
-      </c>
-      <c r="P22" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P22" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Sistemin kaynak belgelerini ya da korpusunu tutan depolar depolamada şifreli.
+c2 [temel] Depo envanteri indeksler, prompt ve yanıt kayıtları, yedekler ve sağlayıcı depoları dahil her AI veri deposunu sayıyor.
+c3 [temel] Envanterdeki depolardan depolamada şifreli olduğu yapılandırma ya da sağlayıcı belgesiyle gösterilenlerin oranı. [%100 (hepsi)]
+c4 [temel] Envanterdeki depolardan anahtar sahibi kayıtlı olanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Anahtar rotasyonu ya da anahtarlara erişim gözden geçirilmiş; tarihli kaydı 12 ay içinde. [≤ 12 ay]</t>
+        </is>
+      </c>
       <c r="Q22" s="6" t="n">
         <v>12</v>
       </c>
@@ -2892,7 +3007,7 @@
       </c>
       <c r="W22" s="6" t="inlineStr">
         <is>
-          <t>Every store in the inventory, including logs, indexes and backups, is encrypted at rest with configuration or provider evidence, and the key holder is recorded for each.</t>
+          <t>c1 and all core checks (c2–c4) met.</t>
         </is>
       </c>
     </row>
@@ -2946,25 +3061,35 @@
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>Sistem için yazılı bir kişisel veri kategori listesi yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>Liste var ama şunlardan en az biri geçerli: kapsamdaki her veri kaynağını kapsamıyor; özel nitelikli verileri içermiyor; veriyle ilgili yerel tanımlayıcıları (ör. TCKN, IBAN) içermiyor; kategori başına muamele tanımlı değil; adı belli bir sahip tarafından onaylanmamış.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>Liste kapsamdaki her veri kaynağını kapsıyor, özel nitelikli verileri ve ilgili yerel tanımlayıcıları içeriyor, kategori başına muamele tanımlıyor ve adı belli bir sahip tarafından onaylanmış.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O23" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve liste 12 ay içinde ya da son veri kaynağı eklendikten sonra (hangisi önce gelirse) gözden geçirilmiş; tarihli gözden geçirme kaydı var.</t>
-        </is>
-      </c>
-      <c r="P23" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P23" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Sistem için tespit edilecek kişisel veri kategorilerinin yazılı listesi var.
+c2 [temel] Kapsamdaki veri kaynaklarından listede karşılığı olanların oranı. [%100 (hepsi)]
+c3 [temel] Liste özel nitelikli kişisel verileri içeriyor.
+c4 [temel] Liste ilgili yerel tanımlayıcıları (ör. TCKN, IBAN) içeriyor.
+c5 [temel] Her kategori için muamele tanımlı; her "izin ver" için yazılı dayanak var.
+c6 [temel] Liste adı belli bir sahip tarafından onaylanmış.
+s1 [sürdürme] Son tarihli gözden geçirme 12 ay içinde ve son veri kaynağı eklenmesinden önce değil.</t>
+        </is>
+      </c>
       <c r="Q23" s="6" t="n">
         <v>12</v>
       </c>
@@ -3001,7 +3126,7 @@
       </c>
       <c r="W23" s="6" t="inlineStr">
         <is>
-          <t>The list covers every in-scope data source, includes special categories and the relevant locale-specific identifiers, defines a treatment per category, and is approved by a named owner.</t>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -3380,25 +3505,35 @@
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>Prompt içeriği kişisel veri için otomatik kontrol olmadan modele ulaşıyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: kanalların yalnız bir kısmı kapsanıyor; ekler kontrol edilmiyor; kontrol tespit edip uyarıyor ama muameleyi uygulamıyor; kullanıcı kayıtlı gerekçe olmadan atlatabiliyor; kayıt kanıtı yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>Ekler dahil her prompt kanalı model çağrısından önce tanımlı muameleyi uyguluyor; kullanıcının her atlatması kayıtlı gerekçe gerektiriyor; o dönemde kullanılan her kanal için son 30 güne ait kayıt var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; atlatmalar ve tespitler 3 ay içinde gözden geçiriliyor, aksiyonlar kayıtlı.</t>
-        </is>
-      </c>
-      <c r="P27" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P27" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir prompt kanalında model çağrısından önce otomatik kişisel veri kontrolü var.
+c2 [temel] Prompt kanallarından kontrolün model çağrısından önce çalıştığı kanalların oranı. [%100 (hepsi)]
+c3 [temel] Serbest metnin yanında ekler de kontrol ediliyor.
+c4 [temel] Kontrol tanımlı muameleyi uyguluyor (yalnız tespit edip uyarmıyor).
+c5 [temel] Kullanıcının her atlatması kayıtlı gerekçe gerektiriyor.
+c6 [temel, QS dışı] Son 30 günde kullanılan kanallardan o döneme ait tespit/muamele kaydı bulunanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Atlatmalar ve tespitler gözden geçirilmiş, aksiyonlar yazılmış; tarihli kaydı 3 ay içinde. [≤ 3 ay]</t>
+        </is>
+      </c>
       <c r="Q27" s="6" t="n">
         <v>3</v>
       </c>
@@ -3433,7 +3568,7 @@
       </c>
       <c r="W27" s="6" t="inlineStr">
         <is>
-          <t>Every prompt channel, including attachments, applies the defined treatment before the model call; any user override requires a logged reason; events from the last 30 days exist for every channel used in that period.</t>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -3590,25 +3725,35 @@
       </c>
       <c r="L29" s="6" t="inlineStr">
         <is>
-          <t>Bir ya da daha fazla AI deposu anonim erişime izin veriyor ya da varsayılan olarak tüm çalışanlara açık.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M29" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: paylaşımlı ya da genel hesapların erişimi var; yetkiler rol tanımlarıyla örtüşmüyor; prompt ve yanıt kayıtları için rol tanımlı değil; hiç erişim gözden geçirmesi yapılmamış.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>Prompt ve yanıt kayıtları dahil her depo için roller tanımlı, erişim yalnız adı belli kimliklerde, yetkiler rol tanımlarıyla örtüşüyor ve son 12 ayda erişim gözden geçirmesi yapılmış.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; erişim gözden geçirmeleri 6 ay içinde yapılıyor ve ayrılan çalışanların erişiminin 2 iş günü içinde kaldırıldığı kayıtlarla gösteriliyor.</t>
-        </is>
-      </c>
-      <c r="P29" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P29" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Her AI veri deposu kimlik doğrulama istiyor ve hiçbiri varsayılan olarak tüm çalışanlara açık değil.
+c2 [temel] Prompt ve yanıt kayıtları dahil depolardan rolleri tanımlı olanların oranı. [%100 (hepsi)]
+c3 [temel] Hiçbir depoya paylaşımlı ya da genel hesabın erişimi yok.
+c4 [temel, QS dışı] Verilmiş yetkilerden rol tanımlarıyla örtüşenlerin oranı. [%100 (hepsi)]
+c5 [temel] Son erişim gözden geçirmesinin (gözden geçiren ve kaldırılan erişimlerle) tarihi son 12 ay içinde. [≤ 12 ay]
+s1 [sürdürme] Son erişim gözden geçirmesinin tarihi 6 ay içinde. [≤ 6 ay]
+s2 [sürdürme] Ayrılan çalışanlardan erişimi 2 iş günü içinde kaldırılanların oranı. [%100 (hepsi)]</t>
+        </is>
+      </c>
       <c r="Q29" s="6" t="n">
         <v>6</v>
       </c>
@@ -3643,7 +3788,7 @@
       </c>
       <c r="W29" s="6" t="inlineStr">
         <is>
-          <t>Every store, including prompt and response logs, has defined roles, only named identities hold access, permissions match the role definitions, and an access review was done in the last 12 months.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -3697,25 +3842,34 @@
       </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
-          <t>Veri girişi kaydedilmiyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>Veri girişi kaydediliyor ama şunlardan en az biri geçerli: dört alandan biri eksik; bazı yollar kaydedilmiyor; sistem yöneticileri girdileri fark edilmeden değiştirip silebiliyor; örnek bir öğe izlenemiyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c4) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>Her yol dört alanı kaydediyor, kayıt deposu listelenen mekanizmalardan en az biriyle korunuyor ve üç örnek öğenin üçü de girdilerine kadar izleniyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c4) karşılanıyor.</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; kayıt bütünlüğü 3 ay içinde doğrulanıyor (ör. özet kontrolü ya da boşluk tespiti) ve kaydı var; kayıt saklama süresi tanımlı süreyle örtüşüyor.</t>
-        </is>
-      </c>
-      <c r="P30" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P30" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir giriş yolunda veri girişi kaydediliyor.
+c2 [temel] Giriş yollarından dört kaynak alanının hepsini kaydedenlerin oranı. [%100 (hepsi)]
+c3 [temel] Kayıt deposu korumalı.
+c4 [temel, QS dışı] Saklanan üç örnek öğe kayıt girdilerine kadar izleniyor. [3/3]
+s1 [sürdürme] Kayıt bütünlüğü doğrulanmış (ör. özet kontrolü ya da boşluk tespiti); tarihli kaydı 3 ay içinde. [≤ 3 ay]
+s2 [sürdürme] Kayıt saklama süresi tanımlı saklama süresiyle örtüşüyor.</t>
+        </is>
+      </c>
       <c r="Q30" s="6" t="n">
         <v>3</v>
       </c>
@@ -3751,7 +3905,7 @@
       </c>
       <c r="W30" s="6" t="inlineStr">
         <is>
-          <t>Every path logs the four fields, the log store is protected by at least one of the listed mechanisms, and all three sampled items are traced to their entries.</t>
+          <t>c1 and all core checks (c2–c4) met.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A2 adım 5: kalan 11 madde kontrol listesine çevrildi — A2 tamam
- CON-ING-02, CON-STO-01, G-RSK-02/03, G-SUP-02/03, G-LIT-02, G-OVS-01, HYG-ING-03/04, IDE-ING-01
- 29 maddenin hepsi kontrol bazlı (182 kontrol); terms.yaml 48 terim; elle yazılmış rubric alanı kalktı
- rehber puanlama notu, README, schema 5.5, şablon, meta güncellendi; çıktılar yeniden üretildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RaFMgY52inRvN44BSaYeeZ
</commit_message>
<xml_diff>
--- a/measurement-tool/output/inceleme-paketi.xlsx
+++ b/measurement-tool/output/inceleme-paketi.xlsx
@@ -1190,25 +1190,32 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>Role özgü AI eğitimi yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: roller modüllerle eşlenmemiş; bir ya da daha fazla rol sahibinin kayıtlı tamamlaması yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c3) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>Her AI rolü bir modülle eşlenmiş ve her güncel rol sahibinin kayıtlı tamamlaması var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c3) karşılanıyor.</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve rol sahipleri 12 ay içinde tazeleme eğitimini tamamlamış.</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Role özgü en az bir yapay zekâ eğitim modülü var.
+c2 [temel] AI rollerinden bir eğitim modülüyle eşlenmiş olanların oranı. [%100 (hepsi)]
+c3 [temel] Güncel rol sahiplerinden modülünü tamamladığı kayıtlı olanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Rol sahiplerinden 12 ay içinde tazeleme eğitimini tamamlayanların oranı. [%100 (hepsi)]</t>
+        </is>
+      </c>
       <c r="Q6" s="6" t="n">
         <v>12</v>
       </c>
@@ -1238,7 +1245,7 @@
       </c>
       <c r="W6" s="6" t="inlineStr">
         <is>
-          <t>Every AI role is mapped to a module and every current role holder has a recorded completion.</t>
+          <t>c1 and all core checks (c2–c3) met.</t>
         </is>
       </c>
     </row>
@@ -1288,25 +1295,32 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>Hiçbir sistem için insan gözetimi tanımlı değil.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: yalnız bazı sistemler için tanımlı; dört unsurdan biri eksik; prosedür hiç uçtan uca işletilmemiş.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c3) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>Her sistem için dört unsur tanımlı (ya da imzalı inceleme-gerekmez kararı var) ve inceleme sınıfı tanımlı her sistemin en az bir kayıtlı uçtan uca işletimi var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c3) karşılanıyor.</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve 6 ay içinde süre sınırında tamamlanan incelemelerin oranı sistem başına ölçülmüş ve kaydedilmiş.</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P7" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir AI sistemi için insan gözetimi tanımlı.
+c2 [temel] Sistemlerden dört gözetim unsurunun hepsi tanımlı ya da imzalı "inceleme gerekmez" kararı olanların oranı. [%100 (hepsi)]
+c3 [temel] İnceleme sınıfı tanımlı sistemlerden en az bir kayıtlı uçtan uca işletimi (gerçek vaka ya da test) olanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Süre sınırında tamamlanan incelemelerin oranı sistem başına ölçülmüş; son tarihli ölçüm 6 ay içinde. [≤ 6 ay]</t>
+        </is>
+      </c>
       <c r="Q7" s="6" t="n">
         <v>6</v>
       </c>
@@ -1343,7 +1357,7 @@
       </c>
       <c r="W7" s="6" t="inlineStr">
         <is>
-          <t>Every system has the four elements defined (or a signed no-review decision), and each system with defined review classes has at least one recorded end-to-end run.</t>
+          <t>c1 and all core checks (c2–c3) met.</t>
         </is>
       </c>
     </row>
@@ -1857,25 +1871,33 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>Hiçbir sistem sınıflandırılmamış.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: yalnız bazı sistemler sınıflandırılmış; gerekçe uygulanan ölçütlere atıf yapmıyor; adı belli imzalayan yok; kuruma uygulanan sektör kuralları dikkate alınmamış.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c4) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>Envanterdeki her sistemin, ölçütlere atıf yapan gerekçeli bir sınıflandırması var, uygulanabilir sektör kuralları dikkate alınmış ve adı belli bir kişi imzalamış.</t>
+          <t>c1 ve tüm temel kontroller (c2–c4) karşılanıyor.</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve sınıflandırmalar 12 ay içinde ve her amaç ya da kullanıcı grubu değişikliğinden sonra yeniden teyit edilmiş, kayıtları var.</t>
-        </is>
-      </c>
-      <c r="P12" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P12" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir AI sisteminin düzenleyici risk sınıflandırması var.
+c2 [temel] Envanterdeki (G-INV-01) sistemlerden sınıflandırma kaydı olanların oranı. [%100 (hepsi)]
+c3 [temel, QS dışı] Sınıflandırmalardan gerekçesi uygulanan ölçütlere (madde ya da ek) atıf yapanların oranı. [%100 (hepsi)]
+c4 [temel] Kuruma uygulanan sektör kuralları listelenmiş ve her sınıflandırma bunların uygulanıp uygulanmadığını belirtiyor.
+s1 [sürdürme] Sınıflandırmalardan 12 ay içinde ve her amaç ya da kullanıcı grubu değişikliğinden sonra yeniden teyit edilenlerin oranı. [%100 (hepsi)]</t>
+        </is>
+      </c>
       <c r="Q12" s="6" t="n">
         <v>12</v>
       </c>
@@ -1908,7 +1930,7 @@
       </c>
       <c r="W12" s="6" t="inlineStr">
         <is>
-          <t>Every inventoried system has a classification with rationale referencing the criteria, applicable sector rules are considered, and a named person signed it.</t>
+          <t>c1 and all core checks (c2–c4) met.</t>
         </is>
       </c>
     </row>
@@ -1958,25 +1980,36 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>Kişisel veri işleyen hiçbir AI sistemi için etki değerlendirmesi yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: yalnız bazı sistemler için değerlendirme var; veri haritası tüm pipeline aşamalarını kapsamıyor; verinin yurt dışına çıktığı noktalar belirlenmemiş; DPO görüşü yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c6) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>Kişisel veri işleyen her AI sisteminin, tüm pipeline aşamalarında veri haritası, belirlenmiş yurt dışı aktarım noktaları, sahipli önlemler ve kayıtlı DPO görüşü içeren değerlendirmesi var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c6) karşılanıyor.</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; önlemler kapanışa kadar izleniyor ve her değerlendirme 12 ay içinde ya da veri kategorisi veya sağlayıcı değişikliğinden sonra güncellenmiş.</t>
-        </is>
-      </c>
-      <c r="P13" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Kişisel veri işleyen en az bir AI sistemi için etki değerlendirmesi var.
+c2 [temel] Kişisel veri işleyen AI sistemlerinden tamamlanmış etki değerlendirmesi olanların oranı. [%100 (hepsi)]
+c3 [temel] Değerlendirmelerden veri haritası altı pipeline aşamasının hepsini kapsayanların oranı. [%100 (hepsi)]
+c4 [temel, QS dışı] Değerlendirmelerden verinin yurt dışına çıktığı her noktayı belirleyenlerin oranı. [%100 (hepsi)]
+c5 [temel, QS dışı] Değerlendirmelerden her önlemin bir sahibi olanların oranı. [%100 (hepsi)]
+c6 [temel] Değerlendirmelerden kayıtlı DPO görüşü olanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Önlemler kapanışa kadar izleniyor (durum ve kapanış tarihi kayıtlı).
+s2 [sürdürme] Değerlendirmelerden 12 ay içinde ya da her veri kategorisi veya sağlayıcı değişikliğinden sonra (hangisi önce gelirse) güncellenenlerin oranı. [%100 (hepsi)]</t>
+        </is>
+      </c>
       <c r="Q13" s="6" t="n">
         <v>12</v>
       </c>
@@ -2010,7 +2043,7 @@
       </c>
       <c r="W13" s="6" t="inlineStr">
         <is>
-          <t>Every AI system processing personal data has an assessment with a data map across all pipeline stages, identified cross-border points, mitigations with owners, and a recorded DPO opinion.</t>
+          <t>c1 and all core checks (c2–c6) met.</t>
         </is>
       </c>
     </row>
@@ -2177,25 +2210,33 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>Üç soru hiçbir sağlayıcı için ele alınmamış.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: yalnız bazı sağlayıcılar için cevaplanmış; üç sorudan biri cevapsız; sınır cevabı yalnız sağlayıcı beyanına dayanıyor; kritik bir sağlayıcı için çıkış planı yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c4) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>Kapsamdaki her sağlayıcı için üç soru kaynaklarıyla cevaplanmış, sınır cevabı çıkış trafiği ya da veri yerleşimi kanıtıyla destekleniyor ve her kritik sağlayıcının çıkış planı ya da alternatif sağlayıcı değerlendirmesi var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c4) karşılanıyor.</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve en az bir kritik sağlayıcının çıkış planı 12 ay içinde işletilmiş (masa başı ya da teknik test), kaydı var.</t>
-        </is>
-      </c>
-      <c r="P15" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P15" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Üç egemenlik sorusu en az bir sağlayıcı ya da barındırma düzeni için ele alınmış.
+c2 [temel] Kapsamdaki sağlayıcılardan üç sorunun hepsi kaynaklarıyla cevaplanmış olanların oranı. [%100 (hepsi)]
+c3 [temel, QS dışı] Sınır cevaplarından yalnız sağlayıcı beyanına değil, çıkış trafiği ya da veri yerleşimi kanıtına dayananların oranı. [%100 (hepsi)]
+c4 [temel] Kritik sağlayıcılardan çıkış planı ya da alternatif sağlayıcı değerlendirmesi olanların oranı. [%100 (hepsi)]
+s1 [sürdürme] En az bir kritik sağlayıcının çıkış planı işletilmiş (masa başı ya da teknik test); tarihli kaydı 12 ay içinde. [≤ 12 ay]</t>
+        </is>
+      </c>
       <c r="Q15" s="6" t="n">
         <v>12</v>
       </c>
@@ -2231,7 +2272,7 @@
       </c>
       <c r="W15" s="6" t="inlineStr">
         <is>
-          <t>All three questions are answered with sources for every provider in scope, the boundary answer is supported by egress or residency evidence, and every critical provider has an exit plan or an alternative-provider assessment.</t>
+          <t>c1 and all core checks (c2–c4) met.</t>
         </is>
       </c>
     </row>
@@ -2281,25 +2322,31 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>Hiçbir sağlayıcı için sözleşme ya da koşullar incelenmemiş ya da beş maddenin hiçbiri yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>Kurum verisiyle kullanılan en az bir sağlayıcıda beş maddeden biri ya da daha fazlası eksik ve sistem sahibinin kayıtlı risk kabulü yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>Kurum verisiyle kullanılan her sağlayıcıda beş maddenin hepsi var ya da eksik her madde için sistem sahibinin imzaladığı ve G-RSK-01'de atıf yapılan bir risk kabulü var.</t>
+          <t>c1 ve tüm temel kontroller (c2) karşılanıyor.</t>
         </is>
       </c>
       <c r="O16" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor ve sağlayıcı koşul değişiklikleri izleniyor: her sağlayıcı için koşulların 12 ay içinde yeniden kontrol edildiğini gösteren kayıt var.</t>
-        </is>
-      </c>
-      <c r="P16" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir sağlayıcının sözleşmesi ya da kabul edilmiş koşulları beş maddeye göre kontrol edilmiş, sonuç kayıtlı.
+c2 [temel] Kurum verisiyle kullanılan sağlayıcılardan beş maddenin her biri var olan ya da eksik her madde için risk kabulü bulunanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Sağlayıcılardan koşulları 12 ay içinde yeniden kontrol edilmiş ve tarihli kaydı olanların oranı. [%100 (hepsi)]</t>
+        </is>
+      </c>
       <c r="Q16" s="6" t="n">
         <v>12</v>
       </c>
@@ -2333,7 +2380,7 @@
       </c>
       <c r="W16" s="6" t="inlineStr">
         <is>
-          <t>Every provider used with organisational data has all five clauses, or each missing clause has a risk acceptance signed by the system owner and referenced in G-RSK-01.</t>
+          <t>c1 and all core checks (c2) met.</t>
         </is>
       </c>
     </row>
@@ -2735,25 +2782,35 @@
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>Dışa açık bir ya da daha fazla akış şifresiz ya da durum bilinmiyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>Dışa açık akışlar şifreli ama şunlardan en az biri geçerli: servisler arası iç akışlar şifresiz; eskimiş protokol sürümleri kabul ediliyor; akış listesi yok; test sonucu sunulamıyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>Listedeki iç ve dış her akış şifreli, eskimiş sürümler reddediliyor ve son 6 aya ait bir test sonucu bunu doğruluyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; sertifika süreleri ve protokol yapılandırması alarmla izleniyor ve test 6 ay içinde tekrarlanıyor.</t>
-        </is>
-      </c>
-      <c r="P20" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P20" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Dış model sağlayıcılarına yapılan çağrılar dahil dışa açık her akış aktarımda şifreli.
+c2 [temel] Her akışın protokolünü gösteren veri akışları listesi var.
+c3 [temel] Listedeki akışlardan, servisler arası iç akışlar dahil, aktarımda şifreli olanların oranı. [%100 (hepsi)]
+c4 [temel] Eskimiş protokol sürümleri her uç noktada reddediliyor.
+c5 [temel, QS dışı] Şifresiz ya da eskimiş protokollü uç nokta olmadığını gösteren son tarama/testin tarihi son 6 ay içinde. [≤ 6 ay]
+s1 [sürdürme] Sertifika süreleri ve protokol yapılandırması alarmla izleniyor.
+s2 [sürdürme] En az iki tarihli test var ve son ikisi arasındaki süre 6 ay'dan uzun değil.</t>
+        </is>
+      </c>
       <c r="Q20" s="6" t="n">
         <v>6</v>
       </c>
@@ -2789,7 +2846,7 @@
       </c>
       <c r="W20" s="6" t="inlineStr">
         <is>
-          <t>Every flow in the list, internal and external, is encrypted, deprecated versions are refused, and a test result from the last 6 months confirms it.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -2839,25 +2896,35 @@
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>AI veri depolarına genel ağdan erişilebiliyor, ayrıştırma yok.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>Şunlardan en az biri geçerli: bazı depolar ayrıştırılmış, diğerleri değil; kurallar envanterde belirtilenden geniş erişime izin veriyor; varsayılan izin; test kaydı yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>Envanterdeki her depo varsayılan red ile ayrıştırılmış, izinli akışlar envanterle örtüşüyor ve tarihli bir test izinsiz bir bileşenin reddedildiğini gösteriyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; kurallar 6 ay içinde envanterle karşılaştırılmış ve kural değişiklikleri kayıtlı onay gerektiriyor.</t>
-        </is>
-      </c>
-      <c r="P21" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s2) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P21" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir AI veri deposu ağ düzeyinde ayrıştırılmış.
+c2 [temel] Depo envanteri her depoya hangi bileşenlerin erişebileceğini gösteriyor.
+c3 [temel] Envanterdeki depolardan varsayılan red ile ayrıştırılmış olanların oranı. [%100 (hepsi)]
+c4 [temel, QS dışı] Ağ kurallarındaki izinli akışlar envanterle örtüşüyor (daha geniş erişim yok).
+c5 [temel, QS dışı] Envanterde olmayan bir bileşenden yapılmış tarihli test bağlantının reddedildiğini gösteriyor.
+s1 [sürdürme] Kurallar envanterle karşılaştırılmış; tarihli kaydı 6 ay içinde. [≤ 6 ay]
+s2 [sürdürme] Bu kurallarda değişiklik kayıtlı bir onay gerektiriyor.</t>
+        </is>
+      </c>
       <c r="Q21" s="6" t="n">
         <v>6</v>
       </c>
@@ -2892,7 +2959,7 @@
       </c>
       <c r="W21" s="6" t="inlineStr">
         <is>
-          <t>Every store in the inventory is segmented with default deny, allowed flows match the inventory, and a dated test shows a non-allowed component is refused.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -3295,25 +3362,34 @@
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>Hata durumunda açık kalıyor (veri işlenmeden geçiyor) ya da davranış bilinmiyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>Fail-closed yapılandırılmış ama hiç test edilmemiş; ya da yalnız bazı hata sınıflarını (ör. erişilemezlik var, desteklenmeyen dil/format yok) veya yalnız bazı yolları kapsıyor.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c3) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>Fail-closed her yolda erişilemezlik, hata/zaman aşımı ve desteklenmeyen dil/format için yapılandırılmış; tarihli test kaydı her sınıfta verinin engellendiğini ya da karantinaya alındığını gösteriyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c3) karşılanıyor.</t>
         </is>
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; test, tespit bileşeninin her değişikliğinde ve en geç 6 ay içinde tekrarlanıyor; karantina olayları alarm üretiyor ve alarmın ele alındığına dair kayıt var.</t>
-        </is>
-      </c>
-      <c r="P25" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s3) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P25" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] En az bir giriş yolunda tespit kontrolü fail-closed yapılandırılmış.
+c2 [temel] Giriş yollarından üç hata sınıfının hepsi için fail-closed yapılandırılmış olanların oranı. [%100 (hepsi)]
+c3 [temel] Tarihli test kaydı üç hata sınıfının her birinde verinin engellendiğini ya da karantinaya alındığını gösteriyor.
+s1 [sürdürme] Son fail-closed testinin tarihi 6 ay içinde. [≤ 6 ay]
+s2 [sürdürme] Test, tespit bileşenindeki her değişiklikten sonra tekrarlanmış (her değişiklik kaydının ardından bir test kaydı var).
+s3 [sürdürme] Karantina olayları alarm üretiyor ve her alarmın ele alınma kaydı var.</t>
+        </is>
+      </c>
       <c r="Q25" s="6" t="n">
         <v>6</v>
       </c>
@@ -3348,7 +3424,7 @@
       </c>
       <c r="W25" s="6" t="inlineStr">
         <is>
-          <t>Fail-closed is configured on every path for unavailability, error/timeout and unsupported language/format, and a dated test record shows data blocked or quarantined in each class.</t>
+          <t>c1 and all core checks (c2–c3) met.</t>
         </is>
       </c>
     </row>
@@ -3398,25 +3474,36 @@
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>Hiç ölçülmemiş.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>Gelişigüzel ölçülmüş; ya da bilinen-cevaplı set kullanılmamış, kategori bazında ölçülmemiş veya sonuç kaydı saklanmamış.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c5) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>HYG-ING-01'deki her kategoriyi kapsayan bilinen-cevaplı setle ölçülmüş; kategori başına recall kaydedilmiş; her kategori eşiğini karşılıyor ya da sahibi ve tarihi belli açık bir aksiyonu var.</t>
+          <t>c1 ve tüm temel kontroller (c2–c5) karşılanıyor.</t>
         </is>
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; ölçüm tespit yapılandırmasının ya da modelinin her değişikliğinde ve en geç 6 ay içinde tekrarlanıyor; sonuçlar zaman serisi olarak saklanıyor.</t>
-        </is>
-      </c>
-      <c r="P26" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1–s3) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P26" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Tespit kalitesi en az bir kez ölçülmüş ve sonucu kayıtlı.
+c2 [temel] Bilinen-cevaplı test seti HYG-ING-01'deki her kategoriyi kapsıyor.
+c3 [temel] Recall kategori başına, tarihli olarak kayıtlı.
+c4 [temel] Sahibi her kategori için bir recall eşiği belirlemiş.
+c5 [temel] Kategorilerden eşiğini karşılayan ya da sahibi ve tarihi belli açık aksiyonu olanların oranı. [%100 (hepsi)]
+s1 [sürdürme] Son ölçümün tarihi 6 ay içinde. [≤ 6 ay]
+s2 [sürdürme] Ölçüm, tespit yapılandırmasının ya da modelinin her değişikliğinden sonra tekrarlanmış.
+s3 [sürdürme] Her ölçüm sonucu saklanıyor; sonuçlar zaman serisi oluşturuyor.</t>
+        </is>
+      </c>
       <c r="Q26" s="6" t="n">
         <v>6</v>
       </c>
@@ -3451,7 +3538,7 @@
       </c>
       <c r="W26" s="6" t="inlineStr">
         <is>
-          <t>Measured with a known-answer set covering every category in HYG-ING-01; per-category recall recorded; each category meets its threshold or has an open action with owner and date.</t>
+          <t>c1 and all core checks (c2–c5) met.</t>
         </is>
       </c>
     </row>
@@ -3618,25 +3705,33 @@
       </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
-          <t>Bir ya da daha fazla giriş yolu kimlik doğrulaması olmadan veri kabul ediyor.</t>
+          <t>Varlık kontrolü (c1) karşılanmıyor.</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>Tüm yollar kimlik doğrulaması istiyor ama şunlardan en az biri geçerli: bir kimlik bilgisi birden çok kaynak ya da kişi tarafından paylaşılıyor; kimlik bilgilerinin süresi dolmuyor ya da yenilenmiyor; test kaydı yok.</t>
+          <t>c1 karşılanıyor; temel kontrollerden (c2–c4) en az biri karşılanmıyor.</t>
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>Her yol kendine ait kimlik bilgileriyle doğrulama istiyor, kimlik bilgileri tanımlı bir sürede doluyor ya da yenileniyor ve tarihli bir test kimliksiz gönderimin reddedildiğini gösteriyor.</t>
+          <t>c1 ve tüm temel kontroller (c2–c4) karşılanıyor.</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
-          <t>2'yi karşılıyor; kaynak kimlik bilgileri 6 ay içinde gözden geçirilmiş ve kullanılmayanlar iptal edilmiş, kaydı var.</t>
-        </is>
-      </c>
-      <c r="P28" s="6" t="inlineStr"/>
+          <t>2 ve tüm sürdürme kontrolleri (s1) karşılanıyor.</t>
+        </is>
+      </c>
+      <c r="P28" s="6" t="inlineStr">
+        <is>
+          <t>c1 [varlık] Her giriş yolu veri kabul etmeden önce kimlik doğrulaması istiyor.
+c2 [temel] Kaynaklardan kendine ait kimlik bilgisiyle doğrulananların oranı. [%100 (hepsi)]
+c3 [temel] Kaynak kimlik bilgileri tanımlı bir sürede doluyor ya da yenileniyor.
+c4 [temel, QS dışı] Tarihli bir test kimliği doğrulanmamış bir gönderimin reddedildiğini gösteriyor.
+s1 [sürdürme] Kaynak kimlik bilgileri gözden geçirilmiş ve kullanılmayanlar iptal edilmiş; tarihli kaydı 6 ay içinde. [≤ 6 ay]</t>
+        </is>
+      </c>
       <c r="Q28" s="6" t="n">
         <v>6</v>
       </c>
@@ -3671,7 +3766,7 @@
       </c>
       <c r="W28" s="6" t="inlineStr">
         <is>
-          <t>Every path requires authentication with individual credentials, credentials expire or rotate on a defined period, and a dated test shows rejection of an unauthenticated submission.</t>
+          <t>c1 and all core checks (c2–c4) met.</t>
         </is>
       </c>
     </row>

</xml_diff>